<commit_message>
update: promptv1.4 and schema v1.2
</commit_message>
<xml_diff>
--- a/data/input/07. SỬ 12. ma trận KSCL lần 1 (1).xlsx
+++ b/data/input/07. SỬ 12. ma trận KSCL lần 1 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\App\matrixquesgen\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2AD11B-AF2D-4D5C-A345-54350CB3D369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274D177D-48D4-4E35-B827-7E93361FAAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="84">
   <si>
     <t>Stt</t>
   </si>
@@ -713,6 +713,363 @@
   </si>
   <si>
     <t>2 (C4a, C4b)</t>
+  </si>
+  <si>
+    <t>Bài 2. Trật tự thế giới trong Chiến tranh lạnh
+==Start of OCR for page 1==
+Học xong bài này, em sẽ:
+◆ Biết cách sưu tầm và sử dụng tư liệu để tìm hiểu về Trật tự thế giới hai cực I-an-ta.
+◆ Trình bày được quá trình hình thành và tồn tại của Trật tự thế giới hai cực I-an-ta.
+◆ Nêu được nguyên nhân dẫn đến sự sụp đổ của Trật tự thế giới hai cực I-an-ta.
+◆ Phân tích được tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta đối với tình hình thế giới.
+Hình 1. Lâu đài Li-va-đi-a thuộc thành phố I-an-ta, Liên Xô
+Hình trên là lâu đài Li-va-đi-a, nơi diễn ra Hội nghị I-an-ta vào năm 1945. Những quyết định của hội nghị này đã tạo cơ sở cho việc thiết lập Trật tự thế giới hai cực I-an-ta. Trật tự này đã trải qua quá trình hình thành và tồn tại như thế nào? Những nguyên nhân nào dẫn đến sự sụp đổ Trật tự thế giới hai cực I-an-ta? Tác động của sự kiện đó đối với tình hình thế giới là gì?
+1 Quá trình hình thành và tồn tại của Trật tự thế giới hai cực I-an-ta
+a) Sự hình thành Trật tự thế giới hai cực I-an-ta
+Hội nghị I-an-ta diễn ra vào giai đoạn cuối của Chiến tranh thế giới thứ hai, từ ngày 4 đến ngày 11 – 2 – 1945, khi phe Đồng minh giành được những thắng lợi quan trọng trên các mặt trận.
+13
+==End of OCR for page 1==
+==Start of OCR for page 2==
+Hình 2. Từ trái sang phải (hàng ghế ngồi): Thủ tướng Anh – U. Sớc-sin, Tổng thống Mỹ – Ph. Ru-dơ-ven, Chủ tịch Hội đồng Bộ trưởng Liên Xô – I. Xta-lin tại Hội nghị I-an-ta
+Hội nghị đưa ra những quyết định về việc kết thúc chiến tranh, tiêu diệt tận gốc phát xít Đức, quân phiệt Nhật Bản và thoả thuận về việc đóng quân, phân chia phạm vi ảnh hưởng ở châu Âu và châu Á sau chiến tranh.
+Ở châu Âu, quân đội Liên Xô chiếm đóng miền Đông nước Đức, Đông Béc-lin và các nước Đông Âu; quân đội Mỹ, Anh và Pháp chiếm đóng miền Tây nước Đức, Tây Béc-lin và các nước Tây Âu. Vùng Đông Âu thuộc phạm vi ảnh hưởng của Liên Xô; vùng Tây Âu thuộc phạm vi ảnh hưởng của Mỹ. Hai nước Áo và Phần Lan trở thành những nước trung lập.
+Ở châu Á, hội nghị chấp nhận những điều kiện để Liên Xô tham chiến tiêu diệt quân phiệt Nhật Bản, bao gồm việc: 1. Duy trì nguyên trạng và công nhận nền độc lập của Mông Cổ; 2. Trả lại cho Liên Xô những quyền lợi bị mất sau chiến tranh Nga – Nhật (1904 – 1905).
+Sau khi Nhật Bản đầu hàng, quân đội Mỹ chiếm đóng Nhật Bản. Ở bán đảo Triều Tiên, quân đội Liên Xô chiếm đóng miền Bắc, quân đội Mỹ chiếm đóng miền Nam, lấy vĩ tuyến 38 làm ranh giới. Trung Quốc cần trở thành một quốc gia thống nhất và dân chủ; Chính phủ Trung Hoa Dân quốc cần cải tổ với sự tham gia của Đảng Cộng sản và các đảng phái dân chủ; trả lại cho Trung Quốc vùng Mãn Châu, đảo Đài Loan và quần đảo Bành Hồ; Mỹ và Liên Xô có quyền lợi ở Trung Quốc.
+Các vùng còn lại ở châu Á (Đông Nam Á, Nam Á, Tây Á) vẫn thuộc phạm vi ảnh hưởng của các nước phương Tây.
+EM CÓ BIẾT ?
+Những quyền lợi của Liên Xô được khôi phục, bao gồm: trả lại phần phía Nam đảo Xa-kha-lin và các đảo lân cận, bốn đảo thuộc quần đảo Cu-rin, quốc tế hoá thương cảng Đại Liên (Trung Quốc), khôi phục việc thuê cảng Lữ Thuận (Trung Quốc) làm căn cứ hải quân, Liên Xô và Trung Quốc cùng khai thác đường sắt Nam Mãn Châu – Đại Liên,…
+Những quyết định của Hội nghị I-an-ta và thoả thuận sau đó của các cường quốc đã trở thành khuôn khổ cho sự thiết lập trật tự thế giới mới, được gọi là Trật tự thế giới hai cực I-an-ta.
+? Trình bày sự hình thành Trật tự thế giới hai cực I-an-ta.
+14
+==End of OCR for page 2==
+==Start of OCR for page 3==
+b) Quá trình tồn tại của Trật tự thế giới hai cực I-an-ta
+Trật tự thế giới hai cực I-an-ta tồn tại từ năm 1945 đến năm 1991, trải qua hai giai đoạn:
+• Giai đoạn từ năm 1945 đến đầu những năm 70 của thế kỉ XX: giai đoạn xác lập và phát triển của Trật tự thế giới hai cực I-an-ta với sự đối đầu giữa một bên là Mỹ, đứng đầu hệ thống tư bản chủ nghĩa và một bên là Liên Xô, đứng đầu hệ thống xã hội chủ nghĩa.
+Trong giai đoạn này, Trật tự thế giới hai cực I-an-ta được định hình với sự thiết lập các khối quân sự đối đầu nhau, tiêu biểu là: Tổ chức Hiệp ước Bắc Đại Tây Dương (NATO) do Mỹ và các nước phương Tây thành lập năm 1949, Tổ chức Hiệp ước Vác-sa-va do Liên Xô và các nước Đông Âu thành lập năm 1955. Hai cực chi phối hầu hết các lĩnh vực phát triển của thế giới.
+Quan hệ quốc tế giữa hai cực trở nên căng thẳng, đặc biệt từ khi bắt đầu cuộc Chiến tranh lạnh với việc Mỹ và Liên Xô tăng cường chạy đua vũ trang, thành lập các liên minh quân sự ở nhiều khu vực trên thế giới. Đồng thời, các cuộc chiến tranh cục bộ, xung đột quân sự đã xảy ra ở nhiều khu vực khác nhau đều có sự hỗ trợ của hai nước đứng đầu hai cực.
+Tuy nhiên, ngay trong giai đoạn này, Trật tự thế giới hai cực I-an-ta bắt đầu bị rạn nứt trước tác động của tình hình thế giới.
+EM CÓ BIẾT ?
+Ở châu Á, chiến tranh Triều Tiên (1950 – 1953), chiến tranh xâm lược Việt Nam của thực dân Pháp (1945 – 1954) và chiến tranh xâm lược Việt Nam của đế quốc Mỹ (1954 – 1975),… là những cuộc chiến tranh cục bộ tiêu biểu. Ở khu vực Trung Đông, chiến tranh Trung Đông giữa I-xra-en và các nước A-rập bắt đầu từ năm 1948 và kéo dài trong nhiều năm.
+TƯ LIỆU. Thắng lợi của cách mạng Trung Quốc năm 1949 đã mở ra bước đột phá đầu tiên, phá vỡ âm mưu khống chế Trung Quốc của Mỹ và những đặc quyền của Liên Xô ở vùng Đông Bắc Trung Quốc. Đồng thời, sự lớn mạnh của các nước Tây Âu, Nhật Bản cũng làm suy giảm vị trí và ảnh hưởng của Mỹ trong hệ thống tư bản chủ nghĩa.
+(Theo Lịch sử thế giới hiện đại, Quyển 2, NXB Đại học Sư phạm, 2016, tr. 94)
+• Giai đoạn từ đầu những năm 70 của thế kỉ XX đến năm 1991: Trật tự thế giới hai cực I-an-ta suy yếu và đi đến sụp đổ.
+Trật tự hai cực I-an-ta có biểu hiện suy yếu khi xu hướng hoà hoãn bắt đầu xuất hiện từ đầu những năm 70 của thế kỉ XX, với việc Liên Xô và Mỹ đạt được thoả thuận bước đầu về hạn chế vũ khí chiến lược, tiến hành cuộc gặp gỡ cấp cao đầu tiên (1972).
+EM CÓ BIẾT ?
+Chuyến thăm chính thức đầu tiên của Tổng thống Mỹ Ních-xơn tới Liên Xô diễn ra vào tháng 5 – 1972. Hai bên đã kí kết nhiều văn kiện quan trọng về hạn chế vũ khí chiến lược, về hợp tác trong các lĩnh vực: khoa học, chinh phục không gian, y học và bảo vệ môi trường,...
+15
+==End of OCR for page 3==
+==Start of OCR for page 4==
+Hình 3. Tổng thống Mỹ Ních-xơn và Tổng Bí thư Ban Chấp hành Trung ương Đảng Cộng sản Liên Xô Brê-giơ-nhép kí các văn kiện (1972)
+Từ nửa sau những năm 80 của thế kỉ XX, Liên Xô và Mỹ đẩy mạnh đối thoại, hợp tác với các cuộc gặp gỡ cấp cao. Hai nước kí kết các văn kiện hợp tác về kinh tế, thương mại, khoa học – kĩ thuật, đặc biệt là thoả thuận về việc thủ tiêu các tên lửa tầm trung ở châu Âu (1987), hạn chế cuộc chạy đua vũ trang. Năm 1989, Liên Xô và Mỹ cùng tuyên bố chấm dứt Chiến tranh lạnh.
+Sự sụp đổ của chủ nghĩa xã hội ở Đông Âu (vào cuối những năm 80 của thế kỉ XX), sự tan rã của Liên Xô (12 – 1991) đã chấm dứt sự tồn tại của Trật tự thế giới hai cực I-an-ta.
+? Khai thác thông tin và tư liệu trong mục, hãy trình bày những nét chính về quá trình tồn tại của Trật tự thế giới hai cực I-an-ta.
+2 Nguyên nhân và tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta
+a) Nguyên nhân sụp đổ
+Sự sụp đổ của Trật tự thế giới hai cực I-an-ta bắt nguồn từ nhiều nguyên nhân.
+Thứ nhất, sự đối đầu căng thẳng đã khiến cho cả hai cực Xô – Mỹ đều bị tốn kém về tài chính, suy giảm thế mạnh kinh tế, phải hạn chế cuộc chạy đua vũ trang để ổn định và củng cố vị thế của mình.
+Thứ hai, từ giữa những năm 70 của thế kỉ XX, cùng với những thay đổi trong quan hệ Xô – Mỹ là những chuyển biến theo hướng hoà dịu trong quan hệ giữa Đông Âu và Tây Âu.
+Thứ ba, sự vươn lên nhanh chóng của các nước trên thế giới nhằm thoát khỏi ảnh hưởng của hai cực, đặc biệt, thắng lợi của phong trào giải phóng dân tộc và sự ra đời của hàng loạt các quốc gia độc lập đã làm thay đổi khuôn khổ của Trật tự thế giới hai cực I-an-ta.
+Thứ tư, sự thay đổi trong cán cân kinh tế thế giới là một yếu tố góp phần làm suy yếu Trật tự thế giới hai cực I-an-ta. Sự vươn lên mạnh mẽ của Nhật Bản và các nước Tây Âu đã tạo ra những trung tâm kinh tế cạnh tranh với Mỹ; sự suy giảm sức mạnh kinh tế của Liên Xô cũng làm cho cán cân kinh tế thế giới thay đổi.
+16
+==End of OCR for page 4==
+==Start of OCR for page 5==
+Thứ năm, cuộc khủng hoảng kinh tế, xã hội và những sai lầm trong công cuộc cải tổ đã làm suy giảm sức mạnh, dẫn tới sự tan rã của Liên Xô – quốc gia đứng đầu hệ thống xã hội chủ nghĩa, cùng với đó là sự sụp đổ của Trật tự thế giới hai cực I-an-ta.
+? Nêu những nguyên nhân dẫn đến sự sụp đổ của Trật tự thế giới hai cực I-an-ta.
+b) Tác động
+Sự sụp đổ của Trật tự thế giới hai cực I-an-ta đã tác động nhiều mặt đến tình hình thế giới.
+Trước hết, sự sụp đổ của Trật tự thế giới hai cực I-an-ta đã mở ra một thời kì phát triển mới trong quan hệ quốc tế, thúc đẩy những xu hướng phát triển mới, đảm bảo lợi ích của các quốc gia, các dân tộc trong quan hệ quốc tế.
+Thứ hai, sự tan rã của Liên Xô đã làm thay đổi so sánh lực lượng với ưu thế tạm thời thuộc về Mỹ. Tuy nhiên, vai trò của các cường quốc khác, các trung tâm kinh tế, các tổ chức quốc tế, khu vực,… ngày càng gia tăng, trong khi sức mạnh của Mỹ cũng suy giảm tương đối.
+Thứ ba, sự sụp đổ của Trật tự thế giới hai cực I-an-ta dẫn đến sự hình thành một trật tự thế giới mới.
+EM CÓ BIẾT ?
+Những khoản thâm hụt ngân sách khổng lồ và nợ nước ngoài gia tăng là những thách thức lớn mà Mỹ phải đối mặt. Năm 1990, thâm hụt ngân sách của Mỹ lên đến 220 tỉ USD (gấp ba lần so với năm 1980), nợ nước ngoài tăng gần 3 000 tỉ USD. Mỹ phải cắt giảm lực lượng quân đội đồn trú ở châu Âu và một số căn cứ quân sự ở các khu vực khác trên thế giới.
+? Phân tích tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta đối với tình hình thế giới.
+LUYỆN TẬP VÀ VẬN DỤNG
+Hãy tóm tắt những nét chính về quá trình hình thành và tồn tại của Trật tự thế giới hai cực I-an-ta.
+Lập sơ đồ tư duy (theo ý tưởng của em) về nguyên nhân và tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta đối với tình hình thế giới.
+Dựa vào tư liệu sưu tầm từ sách, báo, internet và vận dụng những kiến thức đã học, hãy giải thích vì sao sự tồn tại của Trật tự thế giới hai cực I-an-ta không phù hợp với lợi ích chung của cộng đồng quốc tế.
+17
+==End of OCR for page 5==</t>
+  </si>
+  <si>
+    <t>Bài 3. Trật tự thế giới sau Chiến tranh lạnh
+Học xong bài này, em sẽ:
+◆ Nêu được xu thế phát triển chính của thế giới sau Chiến tranh lạnh.
+◆ Trình bày được khái niệm đa cực.
+◆ Nêu được xu thế đa cực trong quan hệ quốc tế sau Chiến tranh lạnh.
+◆ Vận dụng được những hiểu biết về thế giới sau Chiến tranh lạnh để giải thích những vấn đề thời sự trong quan hệ quốc tế.
+Sự kiện Bức tường Béc-lin sụp đổ (11 – 1989) là một trong những biểu tượng cho sự kết thúc của Chiến tranh lạnh. Chiến tranh lạnh kết thúc đã mở ra những xu thế phát triển mới của thế giới. Đó là những xu thế nào? Vì sao xu thế đa cực trở thành xu hướng chính trong quan hệ quốc tế sau Chiến tranh lạnh? Hãy chia sẻ những điều em biết về trật tự thế giới sau Chiến tranh lạnh.
+Hình 1. Người dân Đức trong sự kiện
+Bức tường Béc-lin sụp đổ
+1 Các xu thế phát triển chính của thế giới sau Chiến tranh lạnh
+Chiến tranh lạnh kết thúc đã mở ra một thời kì mới của thế giới với những xu thế phát triển chính: kinh tế là trọng tâm; toàn cầu hoá; đối thoại, hợp tác; đa cực trong quan hệ quốc tế,...
+• Xu thế phát triển lấy kinh tế là trọng tâm
+EM CÓ BIẾT ?
+Từ năm 1986, Việt Nam bắt đầu công cuộc Đổi mới, xây dựng nền kinh tế thị trường định hướng xã hội chủ nghĩa, được xếp trong nhóm những nền kinh tế có tốc độ tăng trưởng cao nhất thế giới, đồng thời gắn kết phát triển kinh tế với tiến bộ và công bằng xã hội.
+Sau Chiến tranh lạnh, hầu hết các quốc gia trên thế giới đều điều chỉnh chiến lược phát triển tập trung vào kinh tế, nhằm tăng cường sức mạnh, tiềm lực quốc gia, đồng thời nâng cao đời sống người dân.
+18
+==End of OCR for page 1==
+==Start of OCR for page 2==
+• Xu thế toàn cầu hoá
+Sự kết thúc của Trật tự thế giới hai cực I-an-ta và Chiến tranh lạnh, cùng với sự phát triển của cách mạng khoa học – công nghệ đã thúc đẩy mạnh mẽ quá trình toàn cầu hoá. Toàn cầu hoá là quá trình gia tăng mạnh mẽ của những mối liên hệ, sự phụ thuộc, tác động lẫn nhau giữa các quốc gia, dân tộc và khu vực trên phạm vi toàn cầu.
+• Xu thế đối thoại, hợp tác trong quan hệ quốc tế
+Nhu cầu ổn định để phát triển kinh tế, đặc biệt là xu thế toàn cầu hoá đã thúc đẩy xu thế đối thoại, cùng hợp tác, thay cho xu thế đối đầu giữa các nước có chế độ chính trị khác nhau trong quan hệ quốc tế. Xu thế đối thoại, hợp tác dựa trên cơ sở hai bên cùng có lợi, tôn trọng lẫn nhau, cùng tồn tại hoà bình đang ngày càng trở thành xu thế chủ yếu trong các mối quan hệ quốc tế.
+? Hãy nêu những xu thế phát triển chính của thế giới sau Chiến tranh lạnh.
+2 Xu thế đa cực trong quan hệ quốc tế
+a) Khái niệm đa cực
+Đa cực là một thuật ngữ trong quan hệ quốc tế dùng để chỉ một trật tự thế giới có sự tham gia của các quốc gia, các trung tâm khác nhau, trong đó không một quốc gia nào có quyền lực áp đảo đối với các quốc gia khác, cũng như chi phối sự phát triển của thế giới.
+Sự hình thành của trật tự thế giới đa cực là một tiến trình lịch sử khách quan với sự nổi lên của các cường quốc, sự gia tăng vai trò của các trung tâm, tổ chức quốc tế, phản ánh tương quan so sánh lực lượng mới trong quan hệ quốc tế sau Chiến tranh lạnh.
+? Trình bày khái niệm đa cực trong quan hệ quốc tế sau Chiến tranh lạnh.
+b) Xu thế đa cực
+Sau Chiến tranh lạnh, xu thế đa cực trở thành một trong những xu thế phát triển chính của thế giới.
+TƯ LIỆU. Nhận định về tình hình thế giới, Đại hội XII của Đảng Cộng sản Việt Nam nêu rõ: "Quá trình toàn cầu hoá và hội nhập quốc tế tiếp tục được đẩy mạnh… Cục diện thế giới theo xu hướng đa cực, đa trung tâm diễn ra nhanh hơn".
+(Đảng Cộng sản Việt Nam, Văn kiện Đại hội đại biểu toàn quốc lần thứ XII,
+NXB Chính trị quốc gia Sự thật, 2016, tr. 16)
+Biểu hiện của xu thế đa cực trước hết là sự gia tăng sức mạnh, tầm ảnh hưởng và vị thế về kinh tế, chính trị, quân sự, đối ngoại,... của các nước lớn như: Trung Quốc, Nga, Ấn Độ, Nhật Bản, một số nước thuộc Liên minh châu Âu (EU),…
+19
+==End of OCR for page 2==
+==Start of OCR for page 3==
+Hình 2. Thành phố Mum-bai – một trong những
+thành phố phát triển nhất Ấn Độ ngày nay
+EM CÓ BIẾT ?
+Mặc dù Mỹ vẫn giữ vị trí số một thế giới về kinh tế và các lĩnh vực như: vốn, khoa học – công nghệ,… nhưng vị thế của nước này đang ngày càng bị giảm dần trước sự nổi lên của các trung tâm khác. Năm 2000, GDP của Mỹ gấp khoảng 12 lần Trung Quốc, nhưng đến năm 2021 chỉ còn gấp khoảng 1,3 lần.
+EM CÓ BIẾT ?
+G20 (gồm các nước nhóm G7, EU, Ác-hen-ti-na, Ô-xtrây-li-a, Bra-xin, Trung Quốc, Mê-hi-cô, Nga, In-đô-nê-xi-a, Ấn Độ, A-rập Xê-út, Nam Phi, Hàn Quốc và Thổ Nhĩ Kỳ), chiếm 2/3 dân số thế giới, 90% GDP toàn cầu và 80% thương mại quốc tế. Được thành lập năm 1999, G20 trở thành trung tâm điều phối các nỗ lực quốc tế nhằm thúc đẩy sự phát triển kinh tế thế giới.
+Cùng với sự phát triển của Trung Quốc, Nga, thế giới còn chứng kiến sự nổi lên của Ấn Độ với mức tăng trưởng kinh tế cao liên tục trong nhiều năm. Nhật Bản và một số nước thuộc Liên minh châu Âu tiếp tục khẳng định tiềm lực kinh tế và vị thế của mình.
+Thứ hai là sự suy giảm sức mạnh tương đối của Mỹ trong tương quan so sánh với các cường quốc khác.
+Thứ ba là vai trò ngày càng gia tăng của các trung tâm, tổ chức kinh tế, tài chính quốc tế, khu vực.
+Sau Chiến tranh lạnh, các tổ chức kinh tế, tài chính khu vực, liên khu vực có vai trò ngày càng lớn đối với sự phát triển của thế giới, tiêu biểu là: Nhóm 20 nền kinh tế lớn nhất thế giới (G20); Diễn đàn Hợp tác Á – Âu (ASEM) gồm các nước thuộc Liên minh châu Âu (EU), các nước ASEAN, Trung Quốc, Nhật Bản, Hàn Quốc.
+Trong xu thế đa cực, Mỹ và Trung Quốc là hai cực có tầm ảnh hưởng lớn, nhưng các nước lớn, các trung tâm kinh tế, chính trị khác cũng đang vươn lên mạnh mẽ để khẳng định vai trò của mình trong quan hệ quốc tế.
+? Nêu những nét chính về xu thế đa cực trong quan hệ quốc tế sau Chiến tranh lạnh.
+LUYỆN TẬP VÀ VẬN DỤNG
+Lập bảng tóm tắt các xu thế phát triển chính của thế giới sau Chiến tranh lạnh.
+Bằng những kiến thức đã học và sưu tầm thêm tư liệu từ sách, báo, internet, em hãy chứng minh nhận định sau: "Hiện nay, cục diện thế giới theo xu hướng đa cực, đa trung tâm diễn ra nhanh hơn". Theo em, xu thế đó mang lại những cơ hội nào cho Việt Nam trong công cuộc phát triển đất nước?
+20
+==End of OCR for page 3==</t>
+  </si>
+  <si>
+    <t>Bài 4. Sự ra đời và phát triển  của Hiệp hội các quốc gia Đông Nam Á
+Học xong bài này, em sẽ:
+◆ Biết cách sưu tầm và sử dụng tài liệu để tìm hiểu quá trình thành lập ASEAN.
+◆ Trình bày được quá trình hình thành và mục đích thành lập của ASEAN.
+◆ Trình bày được quá trình phát triển từ ASEAN 5 đến ASEAN 10.
+◆ Nêu được các giai đoạn phát triển chính của ASEAN (từ năm 1967 đến nay).
+Trong cuốn sách Kì diệu ASEAN – Chất xúc tác cho hoà bình (The ASEAN miracle, A Catalyst for Peace), xuất bản vào dịp kỉ niệm 50 năm thành lập tổ chức ASEAN (1967 – 2017), các tác giả cho rằng thành công của ASEAN là một điều kì diệu và thế giới sẽ trở nên tốt đẹp hơn khi các khu vực đang phát triển khác noi gương sự thành công của ASEAN để tạo ra hoà bình, thịnh vượng. Vì sao ASEAN được đánh giá như một “điều kì diệu”? Hãy chia sẻ những điều em biết về sự hình thành và phát triển của ASEAN.
+Hình 1. Trang bìa cuốn sách “Kì diệu ASEAN – Chất xúc tác cho hoà bình”
+1 Quá trình hình thành và mục đích thành lập tổ chức ASEAN
+a) Quá trình hình thành tổ chức ASEAN
+ASEAN ra đời trong bối cảnh thế giới và khu vực Đông Nam Á có những chuyển biến quan trọng.
+Sau Chiến tranh thế giới thứ hai, xu hướng khu vực hoá trên thế giới bắt đầu xuất hiện và ngày càng trở nên phổ biến. Ở Đông Nam Á, các nước có nhu cầu hợp tác với nhau để cùng phát triển kinh tế, xã hội, đồng thời tạo ra sức mạnh tập thể trong việc ứng phó với sự tranh giành ảnh hưởng giữa các nước lớn đối với khu vực trong bối cảnh Chiến tranh lạnh.
+21
+==End of OCR for page 1==
+==Start of OCR for page 2==
+Đầu những năm 60 của thế kỉ XX, một số tổ chức khu vực được thành lập như: Hiệp hội Đông Nam Á (1961) gồm Ma-lai-xi-a, Phi-líp-pin và Thái Lan; Tổ chức MAPHILINDO (1963) gồm Ma-lai-xi-a, Phi-líp-pin, In-đô-nê-xi-a. Tuy nhiên, các tổ chức này chỉ tồn tại trong một thời gian ngắn, do những bất đồng trong quan hệ song phương giữa một số nước thành viên.
+Vào nửa sau những năm 60, các nước Đông Nam Á ngày càng nhận thức rõ về sự cần thiết của việc hợp tác khu vực, đồng thời quan hệ giữa các nước có những diễn biến thuận lợi cho việc thành lập một tổ chức khu vực.
+Sau các cuộc thảo luận về việc thành lập tổ chức khu vực, ngày 8 – 8 – 1967, tại Băng Cốc (Thái Lan), Ngoại trưởng năm nước: In-đô-nê-xi-a, Ma-lai-xi-a, Phi-líp-pin, Xin-ga-po và Thái Lan đã thông qua Tuyên bố ASEAN (còn gọi là Tuyên bố Băng Cốc), chính thức thành lập Hiệp hội các quốc gia Đông Nam Á (viết tắt theo tiếng Anh là ASEAN).
+Hình 2. Ngoại trưởng năm nước tham gia sáng lập ASEAN (1967)
+? Hãy trình bày quá trình hình thành tổ chức ASEAN.
+b) Mục đích thành lập ASEAN
+TƯ LIỆU. Tuyên bố ASEAN nêu rõ mục đích thành lập của ASEAN:
+Thúc đẩy sự tăng trưởng kinh tế, tiến bộ xã hội và phát triển văn hoá trong khu vực thông qua các nỗ lực chung trên tinh thần bình đẳng và hợp tác nhằm tăng cường cơ sở cho một Cộng đồng các quốc gia Đông Nam Á hoà bình và thịnh vượng.
+Thúc đẩy hoà bình và ổn định khu vực bằng việc tôn trọng công lí và nguyên tắc luật pháp trong quan hệ giữa các quốc gia trong vùng và tuân thủ các nguyên tắc của Hiến chương Liên hợp quốc.
+Thúc đẩy sự cộng tác tích cực và giúp đỡ lẫn nhau trong các vấn đề cùng quan tâm trong các lĩnh vực kinh tế, xã hội, văn hoá, khoa học – kĩ thuật và hành chính,...
+(Theo Tuyên bố ASEAN, Hiệp hội các nước Đông Nam Á (ASEAN), NXB Chính trị quốc gia, 1998, tr. 15 – 16)
+ASEAN được thành lập nhằm mục đích chính là tăng cường hợp tác kinh tế, văn hoá, xã hội, tạo điều kiện cho các nước thành viên phát triển và hội nhập với khu vực, thế giới; phấn đấu để Đông Nam Á trở thành khu vực hoà bình, tự do, thịnh vượng và ASEAN trở thành tổ chức bao gồm tất cả các quốc gia Đông Nam Á.
+? Khai thác thông tin và tư liệu trong mục, hãy trình bày mục đích thành lập ASEAN.
+22
+==End of OCR for page 2==
+==Start of OCR for page 3==
+2 Hành trình phát triển của ASEAN
+a) Từ ASEAN 5 (1967) đến ASEAN 10 (1999)
+Để thực hiện mục tiêu mở rộng thành viên bao gồm tất cả các nước trong khu vực, ASEAN đã trải qua hành trình hơn 30 năm để đưa ASEAN 5 trở thành ASEAN 10.
+1967: ASEAN 5 gồm: Thái Lan, Ma-lai-xi-a, In-đô-nê-xi-a, Xin-ga-po, Phi-líp-pin
+1984: ASEAN 6: Bru-nây gia nhập
+1995: ASEAN 7: Việt Nam gia nhập
+1997: ASEAN 9: Lào và Mi-an-ma gia nhập
+1999: ASEAN 10: Cam-pu-chia gia nhập
+Hình 3. Sơ đồ quá trình phát triển từ ASEAN 5 đến ASEAN 10
+EM CÓ BIẾT ?
+Sự kiện Việt Nam trở thành thành viên thứ bảy của ASEAN là dấu mốc quan trọng trong sự phát triển của ASEAN. Đây không chỉ là sự tăng thêm về số lượng thành viên mà còn đẩy nhanh quá trình thực hiện mục tiêu xây dựng ASEAN trở thành “ngôi nhà chung” của các quốc gia Đông Nam Á.
+Hình 4. Lễ kết nạp Vương quốc Cam-pu-chia là thành viên thứ 10 của ASEAN tại Hà Nội (Việt Nam) năm 1999
+Quá trình mở rộng ASEAN phù hợp với mong muốn, lợi ích của mỗi thành viên, đảm bảo hoà bình, ổn định của cả khu vực, đồng thời nâng cao vị thế của Hiệp hội trên trường quốc tế.
+? Trình bày quá trình phát triển từ ASEAN 5 đến ASEAN 10.
+23
+==End of OCR for page 3==
+==Start of OCR for page 4==
+b) Các giai đoạn phát triển chính của ASEAN (từ năm 1967 đến nay)
+Bảng tóm tắt các giai đoạn phát triển chính của ASEAN
+Các giai đoạn phát triển	Các tuyên bố, hiệp định quan trọng
+1967 – 1976: Giai đoạn khởi đầu, xây dựng nền móng ban đầu, tạo tiền đề cho sự hợp tác ASEAN, tập trung vào hợp tác chính trị – an ninh “xây dựng lòng tin và học cách hoà giải”.	Ra Tuyên bố về Khu vực Hoà bình, Tự do và Trung lập (ZOPFAN, 1971).
+1976 – 1999: Giai đoạn xây dựng quan hệ chính trị ổn định, tạo điều kiện phát triển và hợp tác kinh tế giữa các thành viên; mở rộng ASEAN 5 thành ASEAN 10; từng bước nâng cao uy tín ASEAN trên trường quốc tế, bước đầu mở rộng quan hệ hợp tác, đối thoại với bên ngoài.	– Ra Tuyên bố về sự Hoà hợp ASEAN (Tuyên bố Ba-li I), kí Hiệp ước Thân thiện và Hợp tác ở Đông Nam Á (TAC, 1976),...&lt;br&gt;– Kí Hiệp định khung về tăng cường hợp tác kinh tế ASEAN và thoả thuận về Khu vực Mậu dịch tự do ASEAN (AFTA, 1992), thành lập Diễn đàn khu vực ASEAN (ARF, 1994).
+1999 – 2015: Giai đoạn hoàn thiện cơ cấu tổ chức, tăng cường hợp tác nội khối và ngoại khối về chính trị – an ninh, kinh tế – thương mại và các lĩnh vực khác; khẳng định uy tín, vai trò của ASEAN.	Ra Tuyên bố Ba-li II (2003), công bố Hiến chương ASEAN (2007),...
+2015 đến nay: Thành lập và xây dựng Cộng đồng ASEAN với ba trụ cột: chính trị – an ninh, kinh tế, văn hoá – xã hội; đẩy mạnh hợp tác bên trong ASEAN và bên ngoài ASEAN với các đối tác đối thoại, nâng cao uy tín, vai trò của ASEAN ở khu vực và trên thế giới.	Ra Tuyên bố thành lập Cộng đồng ASEAN (2015), thông qua Tầm nhìn Cộng đồng ASEAN 2025 (2015), Tầm nhìn Cộng đồng ASEAN sau năm 2025 (2020),…
+? Nêu những nét chính về các giai đoạn phát triển của ASEAN từ năm 1967 đến nay.
+LUYỆN TẬP VÀ VẬN DỤNG
+Lập bảng niên biểu về quá trình mở rộng từ ASEAN 5 đến ASEAN 10.
+Có ý kiến cho rằng: Đóng góp quan trọng nhất của ASEAN trong quá trình thành lập và phát triển hơn 50 năm qua là xây dựng được môi trường hoà bình, ổn định ở Đông Nam Á. Em có đồng ý với ý kiến này không? Vì sao?
+Tìm hiểu tư liệu từ sách, báo và internet, hãy viết một bài giới thiệu ngắn gọn về các giai đoạn phát triển của ASEAN từ năm 1967 đến nay.
+24
+==End of OCR for page 4==</t>
+  </si>
+  <si>
+    <t>Bài 5. Cộng đồng ASEAN: Từ ý tưởng đến hiện thực
+Học xong bài này, em sẽ:
+◆ Biết cách sưu tầm và sử dụng tài liệu để tìm hiểu về quá trình hình thành và mục tiêu của Cộng đồng ASEAN.
+◆ Nêu được nét chính về ý tưởng, mục tiêu và kế hoạch xây dựng Cộng đồng ASEAN.
+◆ Trình bày được nội dung ba trụ cột của Cộng đồng ASEAN.
+◆ Nêu được những thách thức và triển vọng của Cộng đồng ASEAN. Có ý thức sẵn sàng tham gia vào các hoạt động xây dựng Cộng đồng ASEAN.
+Tem “Chào mừng Cộng đồng ASEAN” do các hoạ sĩ Việt Nam thiết kế, được phát hành đồng thời tại Việt Nam và các nước ASEAN vào năm 2015. Tem mang thông điệp: “Một Tầm nhìn, một Bản sắc, một Cộng đồng”. Vì sao tất cả các nước thành viên đều chào mừng Cộng đồng ASEAN? Cộng đồng ASEAN được hình thành như thế nào? Hãy chia sẻ những điều em biết về Cộng đồng ASEAN.
+Hình 1. Tem “Chào mừng Cộng đồng ASEAN” năm 2015
+1 Ý tưởng, mục tiêu và kế hoạch xây dựng Cộng đồng ASEAN
+a) Ý tưởng xây dựng Cộng đồng ASEAN
+Ý tưởng xây dựng Cộng đồng ASEAN đã khởi nguồn từ khi ASEAN thành lập. Tuyên bố Băng Cốc (1967) đã nêu ra mục tiêu xây dựng một cộng đồng thịnh vượng và hoà bình ở Đông Nam Á.
+Sau 30 năm phát triển và mở rộng, ASEAN chính thức khẳng định ý tưởng thành lập Cộng đồng ASEAN tại Hội nghị cấp cao ASEAN không chính thức được tổ chức tại Ma-lai-xi-a (1997). Các nước thành viên thông qua văn kiện Tầm nhìn ASEAN 2020, nêu rõ việc xây dựng Cộng đồng ASEAN, định hướng cho sự phát triển trong tương lai của ASEAN.
+TƯ LIỆU 1. Theo Tầm nhìn ASEAN 2020: “Toàn bộ Đông Nam Á sẽ là một cộng đồng ASEAN, nhận thức được các mối liên hệ lịch sử của mình, hiểu rõ di sản văn hoá của mình và gắn bó với nhau bằng một bản sắc chung của khu vực”.
+(Nguồn: Cổng Thông tin ASEAN – Việt Nam)
+25
+==End of OCR for page 1==
+==Start of OCR for page 2==
+Hình 2. Hội nghị cấp cao ASEAN không chính thức tại Ma-lai-xi-a (15 – 12 –1997)
+Với ý tưởng xây dựng Cộng đồng ASEAN, mục tiêu hợp tác về kinh tế, chính trị – an ninh, văn hoá – xã hội giữa các nước thành viên sẽ được phát triển lên một nấc thang mới, đáp ứng nguyện vọng của các quốc gia thành viên về một khu vực Đông Nam Á gắn kết, hữu nghị và hợp tác.
+? Khai thác thông tin và Tư liệu 1 trong mục, hãy nêu những nét chính về ý tưởng xây dựng Cộng đồng ASEAN.
+b) Mục tiêu xây dựng Cộng đồng ASEAN
+Mục tiêu xây dựng Cộng đồng ASEAN là đưa ASEAN trở thành một cộng đồng với ba trụ cột có mức độ liên kết sâu rộng hơn, ràng buộc hơn trên cơ sở pháp lí là Hiến chương ASEAN, đồng thời mở rộng hợp tác với bên ngoài.
+TƯ LIỆU 2. “Cộng đồng ASEAN sẽ được thành lập gồm ba trụ cột là hợp tác chính trị và an ninh, hợp tác kinh tế và hợp tác văn hoá – xã hội được gắn kết chặt chẽ và cùng tăng cường cho mục đích đảm bảo hoà bình, ổn định lâu dài và cùng thịnh vượng trong khu vực.”
+(Trích Tuyên bố Ba-li II (2003), Nguồn: Bộ Ngoại giao)
+? Khai thác thông tin và Tư liệu 2 trong mục, hãy nêu mục tiêu xây dựng Cộng đồng ASEAN.
+c) Kế hoạch xây dựng Cộng đồng ASEAN
+Để thực hiện mục tiêu xây dựng Cộng đồng ASEAN, các nước thành viên đã thông qua kế hoạch triển khai cụ thể trên ba trụ cột: Chính trị – An ninh, Kinh tế, Văn hoá – Xã hội.
+26
+==End of OCR for page 2==
+==Start of OCR for page 3==
+Kế hoạch được nêu rõ trong văn bản “Lộ trình xây dựng Cộng đồng ASEAN (2009 – 2015)”, được thông qua tại Hội nghị cấp cao ASEAN 14 ở Thái Lan (2009), nhằm đưa ASEAN trở thành cộng đồng gắn kết hơn về kinh tế, chính trị – an ninh, có trách nhiệm về xã hội đối với người dân.
+Về quan hệ đối ngoại, ASEAN tăng cường thực hiện các biện pháp mở rộng quan hệ hợp tác với bên ngoài, thông qua cơ chế hợp tác khu vực do ASEAN giữ vai trò chủ đạo.
+Sau sáu năm thực hiện, đến năm 2015, ASEAN đã hoàn thành về cơ bản việc triển khai các kế hoạch xây dựng cộng đồng. Trên cơ sở đó, ngày 22 – 11 – 2015, các nhà lãnh đạo ASEAN đã kí Tuyên bố thành lập Cộng đồng ASEAN, chính thức thành lập Cộng đồng ASEAN kể từ ngày 31 – 12 – 2015.
+Hình 3. Lễ kí Tuyên bố Cu-a-la Lăm-pơ thành lập Cộng đồng ASEAN (2015)
+? Trình bày những nét chính về kế hoạch xây dựng Cộng đồng ASEAN.
+2 Ba trụ cột của Cộng đồng ASEAN
+Ba trụ cột của Cộng đồng ASEAN bao gồm: Cộng đồng Chính trị – An ninh ASEAN (APSC), Cộng đồng Kinh tế ASEAN (AEC) và Cộng đồng Văn hoá – Xã hội ASEAN (ASCC).
+a) Cộng đồng Chính trị – An ninh ASEAN (APSC)
+Cộng đồng Chính trị – An ninh ASEAN được xây dựng trên nền tảng những thành quả hợp tác chính trị – an ninh đã đạt được, nhằm mục tiêu tạo dựng môi trường hoà bình và an ninh ở khu vực, nâng hợp tác chính trị – an ninh lên một nấc thang mới cao hơn và chặt chẽ hơn, trên cơ sở các nguyên tắc cơ bản của ASEAN.
+TƯ LIỆU 3. Kế hoạch Tổng thể xây dựng Cộng đồng Chính trị – An ninh ASEAN (2009 – 2015) bao gồm ba nội dung chính: “Xây dựng một cộng đồng dựa trên các giá trị và chuẩn mực chung; Tạo dựng một khu vực gắn kết, hoà bình và tự cường với trách nhiệm chung đối với an ninh toàn diện; Hướng tới một khu vực năng động và rộng mở với bên ngoài trong một thế giới ngày càng liên kết và tuỳ thuộc”.
+(Nguồn: Cổng Thông tin ASEAN – Việt Nam)
+? Khai thác thông tin và Tư liệu 3 trong mục, hãy trình bày nội dung chính của Cộng đồng Chính trị – An ninh ASEAN.
+27
+==End of OCR for page 3==
+==Start of OCR for page 4==
+b) Cộng đồng Kinh tế ASEAN (AEC)
+Cộng đồng Kinh tế ASEAN là sự tiếp nối các chương trình hợp tác kinh tế của ASEAN trước đây, được mở rộng hơn về phạm vi, mức độ hợp tác kinh tế, thương mại,...
+Hình 4. Các đại biểu tham dự Hội nghị Hội đồng Kinh tế ASEAN lần thứ 18 tại Thái Lan (2019)
+EM CÓ BIẾT ?
+Sau khi AEC thành lập, hợp tác kinh tế giữa các nước ASEAN gia tăng nhanh chóng. Thương mại giữa Việt Nam – ASEAN tăng từ hơn 41 tỉ USD (2016) lên hơn 70 tỉ USD (2021).
+Nội dung chính của Cộng đồng Kinh tế ASEAN bao gồm: tạo ra một thị trường và cơ sở sản xuất chung, trong đó có sự lưu chuyển tự do của hàng hoá, dịch vụ, đầu tư, vốn và lao động có tay nghề; xây dựng khu vực kinh tế có sức cạnh tranh cao, năng động, phát triển đồng đều, hội nhập đầy đủ vào nền kinh tế toàn cầu.
+? Hãy trình bày nội dung chính của Cộng đồng Kinh tế ASEAN.
+c) Cộng đồng Văn hoá – Xã hội ASEAN (ASCC)
+Cộng đồng Văn hoá – Xã hội ASEAN là một khuôn khổ hợp tác chặt chẽ với các quy định và tiêu chuẩn chung để tạo sự hài hoà, bình đẳng và công bằng xã hội, nâng cao ý thức về cộng đồng và bản sắc chung ASEAN.
+TƯ LIỆU 4. Kế hoạch Tổng thể xây dựng Cộng đồng Văn hoá – Xã hội ASEAN (2009) xác định sáu nội dung chính bao gồm: Phát triển con người; Phúc lợi và bảo hiểm xã hội; Bình đẳng xã hội và các quyền; Bảo đảm bền vững về môi trường; Xây dựng bản sắc ASEAN; Thu hẹp khoảng cách phát triển.
+(Theo Bộ Công Thương, Cộng đồng Kinh tế ASEAN 2015, NXB Thế giới, 2016, tr. 10)
+28
+==End of OCR for page 4==
+==Start of OCR for page 5==
+Có nền tảng từ sự phát triển các giá trị văn hoá truyền thống lâu đời, Cộng đồng Văn hoá – Xã hội ASEAN là một trụ cột quan trọng, gắn kết và tạo thuận lợi cho việc xây dựng hai trụ cột Kinh tế và Chính trị – An ninh.
+? Khai thác thông tin và Tư liệu 4 trong mục, hãy trình bày nội dung chính của Cộng đồng Văn hoá – Xã hội ASEAN.
+3 Cộng đồng ASEAN sau năm 2015
+• Tầm nhìn ASEAN sau năm 2015
+Sau khi thành lập Cộng đồng ASEAN, các nước ASEAN tiếp tục đưa ra định hướng cho một giai đoạn phát triển mới sau năm 2015 với nội dung định hướng là tiếp tục củng cố, làm sâu sắc hơn các lĩnh vực hợp tác.
+Hội nghị Cấp cao ASEAN lần thứ 37 tại Hà Nội (2020) đã nhất trí thông qua việc xây dựng Tầm nhìn Cộng đồng ASEAN sau năm 2025, hướng tới việc gắn kết chặt chẽ các nội dung hợp tác trên cả ba trụ cột (Cộng đồng Chính trị – An ninh, Cộng đồng Kinh tế và Cộng đồng Văn hoá – Xã hội), đồng thời bổ sung những nội dung mới như: hợp tác về chuyển đổi số, phát triển nền kinh tế số, kinh tế xanh,...
+Hình 5. Tổng Bí thư, Chủ tịch nước Nguyễn Phú Trọng phát biểu chào mừng khai mạc Hội nghị cấp cao ASEAN lần thứ 37 (2020)
+• Những thách thức và triển vọng của Cộng đồng ASEAN
+Trong quá trình phát triển, Cộng đồng ASEAN phải đối mặt với những thách thức trong nội khối và từ bên ngoài.
+Trong nội khối, những thách thức cơ bản đối với Cộng đồng ASEAN về chính trị là sự đa dạng về chế độ chính trị, tình hình chính trị ở một số nước còn phức tạp, còn tồn tại một số mâu thuẫn trong quan hệ song phương,... Về kinh tế, sự chênh lệch về thu nhập, trình độ phát triển,... giữa các nước gây khó khăn trong hợp tác nội khối; sự tương đồng trong sản xuất một số ngành nghề cũng tạo ra sự cạnh tranh trong xuất khẩu,…
+29
+==End of OCR for page 5==
+==Start of OCR for page 6==
+Bên cạnh đó, những thách thức từ bên ngoài cũng tác động đến Cộng đồng ASEAN như: cạnh tranh ảnh hưởng của các nước lớn đối với khu vực, diễn biến phức tạp của tình hình Biển Đông và tình hình quốc tế; biến đổi khí hậu, ô nhiễm môi trường, dịch bệnh,... Để vượt qua những thách thức, các nước ASEAN đã và đang đẩy nhanh quá trình triển khai các kế hoạch đã đề ra vì lợi ích chung, lâu dài của cả cộng đồng.
+EM CÓ BIẾT ?
+Năm 2021, ASEAN là nền kinh tế lớn thứ năm thế giới với GDP khoảng 3 300 tỉ USD, dự báo đến năm 2030 sẽ trở thành nền kinh tế thứ tư thế giới.
+Về triển vọng, ASEAN sẽ tiếp tục phát triển với mức độ liên kết, hợp tác ngày càng sâu rộng trên cả ba trụ cột, tiếp tục là một trong những khu vực phát triển năng động nhất trên thế giới. Về đối ngoại, ASEAN có quan hệ rộng mở với các đối tác bên ngoài, đồng thời có uy tín, vị thế ngày càng cao trong khu vực và trên thế giới.
+? Nêu những thách thức và triển vọng của Cộng đồng ASEAN.
+LUYỆN TẬP VÀ VẬN DỤNG
+Tóm tắt nét chính về ý tưởng, mục tiêu và kế hoạch xây dựng Cộng đồng ASEAN.
+Lập bảng thống kê (theo gợi ý dưới đây vào vở) về nội dung ba trụ cột của Cộng đồng ASEAN.
+Cộng đồng Chính trị – An ninh	Cộng đồng Kinh tế	Cộng đồng Văn hoá – Xã hội
+?	?	?
+Sưu tầm tư liệu từ sách, báo, internet và vận dụng kiến thức đã học, hãy viết một bài giới thiệu ngắn về những hoạt động của em để góp phần xây dựng Cộng đồng ASEAN vững mạnh, phát triển.
+30
+==End of OCR for page 6==</t>
+  </si>
+  <si>
+    <t>**“Hậu quả tàn khốc của Chiến tranh thế giới thứ hai đã thôi thúc các nước Đồng minh nhất trí về nguyên tắc cần phải thành lập một cơ chế mới, một tổ chức quốc tế mới hoạt động hiệu quả hơn so với Hội Quốc liên(1) để đảm nhận sứ mệnh cao cả gìn giữ hòa bình và ngăn ngừa một cuộc chiến tranh thế giới.... Quyết tâm này được thể hiện rất rõ tại Tuyên bố ở Hội nghị Mát-xcơ-va (tháng 10-1943) và ở Hội nghị Tê-hê-ran (tháng 12-1943) giữa Liên Xô, Anh, Hoa Kỳ và Trung Quốc.... Sau hàng loạt trao đổi trong các năm 1943 - 1944, ngày 25-4-1945, đại biểu của 50 quốc gia đã họp tại Xan Phran-xi-xcô (Hoa Kỳ), soạn thảo và thống nhất thông qua Bản Hiến chương Liên hợp quốc gồm 111 điều vào ngày 25-6-1945.... Ngày 24-10-1945 đánh dấu lịch sử của Liên hợp quốc khi bản Hiến chương được 5 nước thành viên Hội đồng Bảo an cùng hầu hết các quốc gia tham gia ký kết đã phê chuẩn và có hiệu lực.”**  
+(“Liên hợp quốc 70 năm hình thành và phát triển”, Tạp chí Cộng sản, https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/35552/lien-hop-quoc-70-nam-hinh-thanh-va-phat-tr...)[1][3]
+[1](https://tapchicongsan.org.vn)
+[2](https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/to-chuc-quoc-te/lien-hop-quoc-un-3283)
+[3](https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/35552/lien-hop-quoc-70-nam-hinh-thanh-va-phat-trien.aspx)
+[4](https://hcmcpv.org.vn/tin-tuc/viet-nam-va-su-no-luc-khang-dinh-vi-the-trong-to-chuc-lien-hop-quoc-1491884544)
+[5](https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/7754/thong-tin-co-ban-ve-lien-hop-quoc.aspx)
+[6](https://www.tapchicongsan.org.vn/media-story/-/asset_publisher/V8hhp4dK31Gf/content/quan-he-viet-nam-lien-hop-quoc-khoi-dau-hop-tac-moi-vi-mot-tuong-lai-tot-dep-cua-nhan-loai)
+[7](https://www.tapchicongsan.org.vn/the-gioi-van-de-su-kien/-/2018/2946/lien-hop-quoc-trong-boi-canh-quoc-te-moi.aspx)
+[8](https://tapchicongsan.org.vn/web/guest/quoc-phong-an-ninh-oi-ngoai1/-/2018/47141/viet-nam-gia-nhap-lien-hop-quoc--moc-son-lich-su.aspx)
+[9](https://ttdn.vn/nghien-cuu-trao-doi/su-kien-binh-luan/hanh-trinh-80-nam-lien-hop-quoc-tu-qua-khu-den-tuong-lai-113810)
+[10](https://www.studocu.vn/vn/document/hoc-vien-bao-chi-va-tuyen-truyen/quan-he-quoc-te/lien-hop-quoc-doc-mon-quan-he-quoc-te-lien-hop-quoc/61873952)
+[11](https://tapchicongsan.org.vn/web/guest/quoc-phong-an-ninh-oi-ngoai1/-/2018/47741/lien-hop-quoc-va-nhung-dong-gop-cua-viet-nam.aspx)</t>
+  </si>
+  <si>
+    <t>Điều 1 của Hiến chương nêu rõ bốn (04) mục tiêu cơ bản của Liên Hợp quốc là: (1) Duy trì hoà bình và an ninh quốc tế; (2) Thúc đẩy quan hệ hữu nghị giữa các quốc gia trên cơ sở tôn trọng nguyên tắc bình đẳng về quyền lợi giữa các dân tộc và nguyên tắc dân tộc tự quyết; (3) Thực hiện hợp tác quốc tế thông qua giải quyết các vấn đề quốc tế trên các lĩnh vực kinh tế, xã hội, văn hoá và nhân đạo trên cơ sở tôn trọng các quyền con người và quyền tự do cơ bản cho tất cả mọi người, không phân biệt chủng tộc, màu da, ngôn ngữ và tôn giáo; (4) Xây dựng Liên Hợp quốc làm trung tâm điều hoà các nỗ lực quốc tế vì các mục tiêu chung. Và 6 nguyên tắc hoạt động chủ yếu của Liên Hợp quốc là: (1) Bình đẳng về chủ quyền quốc gia; (2) Tôn trọng toàn vẹn lãnh thổ và độc lập chính trị quốc gia; (3) Cấm đe doạ sử dụng vũ lực hoặc sử dụng vũ lực trong quan hệ quốc tế; (4) Không can thiệp vào công việc nội bộ các nước; (5) Tôn trọng các nghĩa vụ quốc tế và luật pháp quốc tế; và (6) Giải quyết các tranh chấp quốc tế bằng biện pháp hoà bình.”
+(“Thông tin cơ bản về Liên hợp quốc”, Tạp chí Cộng sản, https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/7754/thong-tin-co-ban-ve-lien-hop-quoc.aspx)[1]</t>
+  </si>
+  <si>
+    <t>Chiến tranh thế giới thứ II kết thúc, phe Trục phát xít Đức - Italia - Nhật Bản thất bại hoàn toàn, Liên Xô và các nước Đồng minh giành thắng lợi. Cuộc chiến này đã làm thay đổi căn bản tương quan sức mạnh giữa các nước, trung tâm quyền lực trong quan hệ quốc tế, đưa đến hình thành một trật tự thế giới mới cả về chính trị và kinh tế.
+Hội nghị nguyên thủ ba nước là Anh, Mỹ và Liên Xô tại Teheran (tháng 10 - 1943), đặc biệt các cuộc đàm phán tại Yalta (tháng 2 - 1945) và Posdam (tháng 7-8 năm 1945) đã sắp xếp lại quyền lực trong quan hệ quốc tế và từ đây thế giới hình thành nên hệ thống hay trật tự thế giới hai cực, một cực do Liên Xô đứng đầu và cực kia do Mỹ đứng đầu đối nghịch nhau về ý thức hệ chính trị - tư tưởng, kinh tế và quân sự.</t>
+  </si>
+  <si>
+    <t>Trong thời kỳ này, mặc dù nước Anh trong hai phần đầu của thế kỷ XIX, nước Mỹ từ đầu thế kỷ XX có sức mạnh vượt trội, nhưng không thể thiết lập được một thế giới đơn cực bởi sự nổi lên của các cường quốc mới như Pháp, Đức, Nhật và nhất là Liên Xô sau đó. Trật tự thế giới hai cực được hình thành sau Hội nghị Yalta năm 1945 và kết thúc vào năm 1991. Đặc trưng của giai đoạn này là siêu cường Liên Xô và Mỹ đối đầu nhau về ý thức và quân sự. Thế giới bị phân chia thành hai phe, phe XHCN do Liên Xô dẫn dắt và phe TBCN do Mỹ đứng đầu. Hầu hết các quan hệ quốc tế  bị chi phối bởi tư duy của Chiến tranh Lạnh, cho dù hệ thống hay trật tự quốc tế dựa trên luật lệ đã được hình thành, điển hình là hệ thống Liên hợp quốc. Còn trật tự thế giới đơn cực hay khoảnh khắc của trật tự đơn cực do Mỹ nắm vai trò chủ đạo được thiết lập từ khi Liên Xô tan rã đến cuối thập niên đầu thế kỷ XXI.</t>
+  </si>
+  <si>
+    <t>“Chiến tranh lạnh kết thúc, thế giới chuyển từ thời đại địa chính trị sang thời đại của địa kinh tế, mà ở đó cuộc đua tranh giữa các quốc gia dù vẫn được xác định bởi ‘logic của xung đột’ nhưng thông qua ‘ngôn ngữ thương mại’. Theo quan điểm của Luttwak, địa kinh tế là hình thức mới của sự cạnh tranh sức mạnh giữa các quốc gia sau chiến tranh lạnh. Ông cho rằng, chính trị quốc tế thời kỳ hậu chiến tranh lạnh mặc dù vẫn bị chi phối bởi cạnh tranh sức mạnh giữa các nhà nước nhưng chiến trường chủ yếu là kinh tế thay vì quân sự, phương tiện ưa thích được các nhà nước sử dụng để theo đuổi các mục tiêu đối kháng nhau sẽ là kinh tế hơn là quân sự.” (“Mối quan hệ giữa địa chính trị và địa kinh tế - Lý luận và thực tiễn”, Tạp chí Lý luận chính trị, 26/09/2019, https://lyluanchinhtri.vn/moi-quan-he-giua-dia-chinh-tri-va-dia-kinh-te-ly-luan-va-thuc-tien-431.html”)</t>
+  </si>
+  <si>
+    <t>Trong khi đó, sau Chiến tranh Thế giới thứ II, các trào lưu hình thành “chủ nghĩa khu vực” trên thế giới đã xuất hiện và cùng với nó là sự ra đời của Cộng đồng Kinh tế Châu Âu (EEC); Khu vực Thương mại Tự do Mỹ Latin (LAFTA); Thị trường chung Trung Mỹ (CACM)....Việc thành lập các tổ chức khu vực này đã tác động đến việc hình thành ASEAN.
+Từ kinh nghiệm của EEC, các nước Đông Nam Á đều thấy rằng việc hình thành các tổ chức khu vực sẽ giúp thúc đẩy sự tăng trưởng kinh tế thông qua tăng cường hợp tác kinh tế, buôn bán và phân công lao động.
+Về mặt chính trị, các tổ chức khu vực giúp củng cố tình đoàn kết khu vực và giúp các nước vừa và nhỏ có tiếng nói mạnh mẽ hơn trong các vấn đề quốc tế. Còn về mặt xã hội, chủ nghĩa khu vực có thể đưa ra các phương hướng hợp tác để giải quyết có hiệu quả các vấn đề đặt ra cho các nước thành viên.
+Sau nhiều cuộc thảo luận, ngày 8/8/1967, Bộ trưởng Ngoại giao các nước Indonesia, Thái Lan, Philippines, Singapore và Phó Thủ tướng Malaysia ký tại Bangkok bản Tuyên bố thành lập Hiệp hội các quốc gia Đông Nam Á (ASEAN).
+Từ 5 nước thành viên ban đầu, đến nay ASEAN đã có 10 quốc gia thành viên, gồm Indonesia, Thái Lan, Philippines, Singapore, Malaysia, Bruney (năm 1984), Việt Nam (năm1995), Lào (năm 1997), Myanmar (năm 1997) và Campuchia (năm1999).
+ASEAN có diện tích 4,5 triệu km2, dân số khoảng 575 triệu người và tổng sản phẩm quốc nội (GDP) đạt 2.487 tỷ USD (ước tính năm 2009).
+Thực tiễn đã chứng minh rằng, một Đông Nam Á thống nhất đã thúc đẩy cho hợp tác và vị thế ASEAN ngày càng lớn mạnh, là tiền đề quan trọng để ASEAN trở thành một cộng đồng.</t>
+  </si>
+  <si>
+    <t>Những cột mốc phát triển quan trọng
++ Tuyên bố ASEAN:
+Ngày 8/8/1967, tại Bangkok, Thái Lan, Bộ trưởng phụ trách các vấn đề chính trị kiêm Bộ trưởng Ngoại giao Indonesia, Phó Thủ tướng Malaysia, Bộ trưởng Ngoại giao Philippines, Bộ trưởng Ngoại giao Singapore và Bộ trưởng Ngoại giao Thái Lan đã ra Tuyên bố ASEAN.
+Đây là Tuyên bố thành lập Hiệp hội các quốc gia Đông Nam Á với mục tiêu đẩy mạnh tăng trưởng kinh tế, tiến bộ xã hội, phát triển văn hóa; tăng cường hợp tác, giúp đỡ lẫn nhau cũng như thúc đẩy hòa bình, ổn định trong khu vực.
++ Tuyên bố về khu vực hòa bình, tự do và trung lập:
+Ngày 27/11/1971, tại Kuala Lumpur, Malaysia, Bộ trưởng Ngoại giao Indonesia, Malaysia, Philippines, Xingapo và Đặc phái viên của Hội đồng Hành pháp Quốc gia Thái Lan đã ký và công bố “Tuyên bố về khu vực hòa bình, tự do và trung lập ở Đông Nam Á”- Tuyên bố ZOPFAN.
+Tuyên bố quan trọng này đã định ra các mục tiêu cơ bản và lâu dài của ASEAN là xây dựng Đông Nam á thành một khu vực hòa bình, tự do và trung lập, không có sự can thiệp dưới bất cứ hình thức nào của các cường quốc bên ngoài.
++ Hiệp ước Thân thiện và Hợp tác Đông Nam Á:
+Ngày 24/2/1976, tại Bali, Indonesia, nguyên thủ quốc gia các nước ASEAN ký Hiệp ước Thân thiện và Hợp tác ở Đông Nam Á (Hiệp ước Bali).Hiệp ước nhằm thúc đẩy hòa bình vĩnh viễn, tình hữu nghị và hợp tác lâu bền giữa nhân dân các bên tham gia Hiệp ước, góp phần tăng cường sức mạnh, tình đoàn kết và quan hệ chặt chẽ hơn giữa các nước Đông Nam Á.</t>
+  </si>
+  <si>
+    <t>Ngay sau khi chiến tranh chấm dứt, các tổ chức phát triển của Liên hợp quốc đã nhanh chóng hỗ trợ Việt Nam khắc phục hậu quả chiến tranh, tái thiết đất nước và vượt qua những khó khăn kinh tế - xã hội hết sức nặng nề. Liên hợp quốc là cầu nối để Việt Nam tiếp cận nguồn viện trợ nước ngoài và từng bước phá vỡ thế bao vây, cấm vận. Trong giai đoạn đổi mới, Liên hợp quốc tiếp tục hỗ trợ Việt Nam phát triển nguồn lực khoa học - kỹ thuật, nâng cao năng lực, hoàn thiện khuôn khổ pháp luật, chính sách, xóa đói, giảm nghèo. Nguồn vốn, tri thức, kinh nghiệm từ hệ thống Liên hợp quốc không chỉ góp phần giúp Việt Nam thúc đẩy công nghiệp hóa, hiện đại hóa đất nước, đạt nhiều thành tựu phát triển kinh tế - xã hội và thực hiện các mục tiêu phát triển toàn cầu, mà còn đóng vai trò quan trọng trong tiến trình hội nhập quốc tế của Việt Nam. 
+Về phía mình, Việt Nam không ngừng khẳng định vai trò chủ động và đóng góp tích cực vào các hoạt động của Liên hợp quốc, chia sẻ sâu sắc những giá trị cốt lõi của tổ chức này. Từ một nước nhận viện trợ của Liên hợp quốc, Việt Nam chuyển mình, từng bước trở thành thành viên tin cậy, hiệu quả của Liên hợp quốc, là nước đóng góp lớn thứ 49 cho ngân sách của Liên hợp quốc, tham gia ngày càng sâu rộng trên cả ba trụ cột chính: hòa bình - an ninh, hợp tác phát triển và quyền con người.</t>
+  </si>
+  <si>
+    <t>Từ tro tàn của Chiến tranh thế giới lần thứ hai, ngày 24-10-1945, Liên hợp quốc được thành lập với sứ mệnh cao cả là “cứu các thế hệ mai sau khỏi thảm họa chiến tranh đã gây ra đau thương tột cùng cho nhân loại hai lần trong một đời người”. Sự ra đời của Liên hợp quốc là bước ngoặt quan trọng trong lịch sử với cam kết ngăn chặn, loại bỏ các mối đe dọa đối với hòa bình và an ninh quốc tế, các hành vi xâm lược, thúc đẩy giải quyết tranh chấp bằng biện pháp hòa bình.
+Hiến chương Liên hợp quốc là văn kiện nền tảng đặt ra các nguyên tắc cốt lõi mà mọi quốc gia thành viên phải tuân thủ, là khuôn khổ điều chỉnh hành vi của các quốc gia trong suốt gần 80 năm qua và tạo nền tảng cho hệ thống luật pháp quốc tế hiện đại. Đặc biệt, lần đầu tiên trong lịch sử nhân loại, hành vi đe dọa sử dụng vũ lực hoặc sử dụng vũ lực nhằm xâm phạm sự toàn vẹn lãnh thổ và độc lập chính trị của một quốc gia hoặc gây tổn hại đến hòa bình và an ninh quốc tế, bị nghiêm cấm theo Điều 2 của Hiến chương Liên hợp quốc.</t>
+  </si>
+  <si>
+    <t>Hội nghị I-an-ta diễn ra từ ngày 4 đến ngày 11-2-1945 đã đưa ra những quyết định quan trọng về việc kết thúc chiến tranh và thỏa thuận về việc đóng quân, phân chia phạm vi ảnh hưởng ở châu Âu và châu Á. Những quyết định này cùng với những thỏa thuận sau đó của các cường quốc đã trở thành khuôn khổ cho sự thiết lập trật tự thế giới mới, gọi là Trật tự thế giới hai cực I-an-ta. Trong quá trình tồn tại, trật tự này được định hình với sự thiết lập các khối quân sự đối đầu nhau, tiêu biểu là Tổ chức Hiệp ước Bắc Đại Tây Dương (NATO) và Tổ chức Hiệp ước Vác-sa-va</t>
+  </si>
+  <si>
+    <t>Tuyên bố Kuala Lupur về việc hình thành Cộng đồng ASEAN vào ngày 31-12-2015 khẳng định cam kết của các nước thành viên đối với Hiến chương ASEAN, phản ánh mong muốn và ý chí tập thể nhằm chung sống trong một khu vực hòa bình, an ninh và ổn định dài lâu, tăng trưởng kinh tế bền vững, thịnh vượng chung và tiến bộ xã hội,… đánh dấu một bước ngoặt lịch sử mới trong quá trình phát triển của ASEAN, phản ánh được sự lớn mạnh của ASEAN sau gần 48 năm hình thành, phát triển và vươn lên trở thành một Cộng đồng liên kết chặt chẽ trên cả 3 trụ cột là chính trị - an ninh, kinh tế và văn hóa - xã hội với vị thế ngày càng cao ở cả khu vực và thế giới.
+Các nhà lãnh đạo ASEAN coi việc hình thành Cộng đồng ASEAN 2015 là dấu mốc lịch sử trong tiến trình liên kết khu vực, đánh dấu bước chuyển mình chiến lược của ASEAN và khởi đầu cho một giai đoạn phát triển mới ở tầm cao hơn của ASEAN. Đồng thời nhấn mạnh, xây dựng Cộng đồng ASEAN là một tiến trình liên tục; nhất trí rằng, ASEAN cần tiếp tục củng cố và đưa liên kết ASEAN lên tầm cao mới trên cơ sở tiếp nối và phát huy các thành tựu đã đạt được.
+Theo đó, các nhà lãnh đạo ASEAN đã thông qua Tầm nhìn Cộng đồng ASEAN 2025 và ba Kế hoạch Tổng thể triển khai Tầm nhìn trên 3 trụ cột với chủ đề “ASEAN 2025: cùng vững vàng tiến bước” định hướng và tạo cơ sở, khuôn khổ cho liên kết của ASEAN trong mười năm tới. Các nhà lãnh đạo cam kết triển khai hiệu quả các văn kiện này; đồng thời nhất trí, cần tiếp tục triển khai hiệu quả Kế hoạch Tổng thể về Kết nối và Sáng kiến Liên kết ASEAN về thu hẹp khoảng cách phát triển để hỗ trợ cho tiến trình xây dựng Cộng đồng.</t>
+  </si>
+  <si>
+    <t>Tài liệu bổ sung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“Chiến tranh lạnh” kết thúc, trật tự hai cực biểu hiện cuộc đối đầu Đông – Tây khốc liệt của thế giới đã đi đến điểm kết. Song, trật tự thế giới mới vẫn còn đang trong quá trình hình thành. Dựa vào thực lực kinh tế, chính trị và quân sự của mình, Mỹ không từ bỏ mục đích bá chủ thế giới. Tuy nhiên, sự phát triển không ngừng của Nhật Bản, Tây Âu; sự vươn lên mạnh mẽ của Trung Quốc; những cuộc đấu tranh mạnh mẽ nhằm củng cố, bảo vệ độc lập, chủ quyền của các nước thuộc “thế giới thứ ba” dưới nhiều hình thức, biện pháp để chống lại sự can thiệp và ảnh hưởng của các nước lớn… đã tạo ra những tương quan lực lượng không nhỏ đối với Mỹ. Điều này cho thấy, thế giới hậu lưỡng cực đang hướng tới xác lập một trật tự mới với nhiều hướng khác nhau: đơn cực, đa cực, nhất siêu đa cường...
+Sự kết thúc của “Chiến tranh lạnh” tuy không mở ra kỷ nguyên mới hòa bình và thịnh vượng như nhân loại tiến bộ mong đợi vì những xung đột sắc tộc, mâu thuẫn tôn giáo và các cuộc chiến tranh cục bộ ở nhiều khu vực vẫn diễn ra triền miên, song đã tạo ra những điều kiện khiến cho xu thế hòa dịu, hòa hoãn trở nên chiếm ưu thế trong quan hệ giữa các quốc gia, dân tộc trên thế giới; tạo những tiền đề cho đa cực hóa các mối quan hệ- một điều kiện quan trọng dẫn đến hình thành xu thế đa dạng hóa, đa phương hóa, hội nhập khu vực và quốc tế trong quan hệ quốc tế hiện nay.
+https://www.tapchicongsan.org.vn/web/guest/nghien-cu/-/2018/3089/xu-the-da-dang-hoa%2C-da-phuong-hoa%2C-hoi-nhap-khu-vuc-va-quoc-te-hien-nay.aspx </t>
   </si>
   <si>
     <t>Bài 1. Liên Hợp Quốc
@@ -846,296 +1203,12 @@
 12
 ==End of OCR for page 7==</t>
   </si>
-  <si>
-    <t>Bài 2. Trật tự thế giới trong Chiến tranh lạnh
-==Start of OCR for page 1==
-Học xong bài này, em sẽ:
-◆ Biết cách sưu tầm và sử dụng tư liệu để tìm hiểu về Trật tự thế giới hai cực I-an-ta.
-◆ Trình bày được quá trình hình thành và tồn tại của Trật tự thế giới hai cực I-an-ta.
-◆ Nêu được nguyên nhân dẫn đến sự sụp đổ của Trật tự thế giới hai cực I-an-ta.
-◆ Phân tích được tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta đối với tình hình thế giới.
-Hình 1. Lâu đài Li-va-đi-a thuộc thành phố I-an-ta, Liên Xô
-Hình trên là lâu đài Li-va-đi-a, nơi diễn ra Hội nghị I-an-ta vào năm 1945. Những quyết định của hội nghị này đã tạo cơ sở cho việc thiết lập Trật tự thế giới hai cực I-an-ta. Trật tự này đã trải qua quá trình hình thành và tồn tại như thế nào? Những nguyên nhân nào dẫn đến sự sụp đổ Trật tự thế giới hai cực I-an-ta? Tác động của sự kiện đó đối với tình hình thế giới là gì?
-1 Quá trình hình thành và tồn tại của Trật tự thế giới hai cực I-an-ta
-a) Sự hình thành Trật tự thế giới hai cực I-an-ta
-Hội nghị I-an-ta diễn ra vào giai đoạn cuối của Chiến tranh thế giới thứ hai, từ ngày 4 đến ngày 11 – 2 – 1945, khi phe Đồng minh giành được những thắng lợi quan trọng trên các mặt trận.
-13
-==End of OCR for page 1==
-==Start of OCR for page 2==
-Hình 2. Từ trái sang phải (hàng ghế ngồi): Thủ tướng Anh – U. Sớc-sin, Tổng thống Mỹ – Ph. Ru-dơ-ven, Chủ tịch Hội đồng Bộ trưởng Liên Xô – I. Xta-lin tại Hội nghị I-an-ta
-Hội nghị đưa ra những quyết định về việc kết thúc chiến tranh, tiêu diệt tận gốc phát xít Đức, quân phiệt Nhật Bản và thoả thuận về việc đóng quân, phân chia phạm vi ảnh hưởng ở châu Âu và châu Á sau chiến tranh.
-Ở châu Âu, quân đội Liên Xô chiếm đóng miền Đông nước Đức, Đông Béc-lin và các nước Đông Âu; quân đội Mỹ, Anh và Pháp chiếm đóng miền Tây nước Đức, Tây Béc-lin và các nước Tây Âu. Vùng Đông Âu thuộc phạm vi ảnh hưởng của Liên Xô; vùng Tây Âu thuộc phạm vi ảnh hưởng của Mỹ. Hai nước Áo và Phần Lan trở thành những nước trung lập.
-Ở châu Á, hội nghị chấp nhận những điều kiện để Liên Xô tham chiến tiêu diệt quân phiệt Nhật Bản, bao gồm việc: 1. Duy trì nguyên trạng và công nhận nền độc lập của Mông Cổ; 2. Trả lại cho Liên Xô những quyền lợi bị mất sau chiến tranh Nga – Nhật (1904 – 1905).
-Sau khi Nhật Bản đầu hàng, quân đội Mỹ chiếm đóng Nhật Bản. Ở bán đảo Triều Tiên, quân đội Liên Xô chiếm đóng miền Bắc, quân đội Mỹ chiếm đóng miền Nam, lấy vĩ tuyến 38 làm ranh giới. Trung Quốc cần trở thành một quốc gia thống nhất và dân chủ; Chính phủ Trung Hoa Dân quốc cần cải tổ với sự tham gia của Đảng Cộng sản và các đảng phái dân chủ; trả lại cho Trung Quốc vùng Mãn Châu, đảo Đài Loan và quần đảo Bành Hồ; Mỹ và Liên Xô có quyền lợi ở Trung Quốc.
-Các vùng còn lại ở châu Á (Đông Nam Á, Nam Á, Tây Á) vẫn thuộc phạm vi ảnh hưởng của các nước phương Tây.
-EM CÓ BIẾT ?
-Những quyền lợi của Liên Xô được khôi phục, bao gồm: trả lại phần phía Nam đảo Xa-kha-lin và các đảo lân cận, bốn đảo thuộc quần đảo Cu-rin, quốc tế hoá thương cảng Đại Liên (Trung Quốc), khôi phục việc thuê cảng Lữ Thuận (Trung Quốc) làm căn cứ hải quân, Liên Xô và Trung Quốc cùng khai thác đường sắt Nam Mãn Châu – Đại Liên,…
-Những quyết định của Hội nghị I-an-ta và thoả thuận sau đó của các cường quốc đã trở thành khuôn khổ cho sự thiết lập trật tự thế giới mới, được gọi là Trật tự thế giới hai cực I-an-ta.
-? Trình bày sự hình thành Trật tự thế giới hai cực I-an-ta.
-14
-==End of OCR for page 2==
-==Start of OCR for page 3==
-b) Quá trình tồn tại của Trật tự thế giới hai cực I-an-ta
-Trật tự thế giới hai cực I-an-ta tồn tại từ năm 1945 đến năm 1991, trải qua hai giai đoạn:
-• Giai đoạn từ năm 1945 đến đầu những năm 70 của thế kỉ XX: giai đoạn xác lập và phát triển của Trật tự thế giới hai cực I-an-ta với sự đối đầu giữa một bên là Mỹ, đứng đầu hệ thống tư bản chủ nghĩa và một bên là Liên Xô, đứng đầu hệ thống xã hội chủ nghĩa.
-Trong giai đoạn này, Trật tự thế giới hai cực I-an-ta được định hình với sự thiết lập các khối quân sự đối đầu nhau, tiêu biểu là: Tổ chức Hiệp ước Bắc Đại Tây Dương (NATO) do Mỹ và các nước phương Tây thành lập năm 1949, Tổ chức Hiệp ước Vác-sa-va do Liên Xô và các nước Đông Âu thành lập năm 1955. Hai cực chi phối hầu hết các lĩnh vực phát triển của thế giới.
-Quan hệ quốc tế giữa hai cực trở nên căng thẳng, đặc biệt từ khi bắt đầu cuộc Chiến tranh lạnh với việc Mỹ và Liên Xô tăng cường chạy đua vũ trang, thành lập các liên minh quân sự ở nhiều khu vực trên thế giới. Đồng thời, các cuộc chiến tranh cục bộ, xung đột quân sự đã xảy ra ở nhiều khu vực khác nhau đều có sự hỗ trợ của hai nước đứng đầu hai cực.
-Tuy nhiên, ngay trong giai đoạn này, Trật tự thế giới hai cực I-an-ta bắt đầu bị rạn nứt trước tác động của tình hình thế giới.
-EM CÓ BIẾT ?
-Ở châu Á, chiến tranh Triều Tiên (1950 – 1953), chiến tranh xâm lược Việt Nam của thực dân Pháp (1945 – 1954) và chiến tranh xâm lược Việt Nam của đế quốc Mỹ (1954 – 1975),… là những cuộc chiến tranh cục bộ tiêu biểu. Ở khu vực Trung Đông, chiến tranh Trung Đông giữa I-xra-en và các nước A-rập bắt đầu từ năm 1948 và kéo dài trong nhiều năm.
-TƯ LIỆU. Thắng lợi của cách mạng Trung Quốc năm 1949 đã mở ra bước đột phá đầu tiên, phá vỡ âm mưu khống chế Trung Quốc của Mỹ và những đặc quyền của Liên Xô ở vùng Đông Bắc Trung Quốc. Đồng thời, sự lớn mạnh của các nước Tây Âu, Nhật Bản cũng làm suy giảm vị trí và ảnh hưởng của Mỹ trong hệ thống tư bản chủ nghĩa.
-(Theo Lịch sử thế giới hiện đại, Quyển 2, NXB Đại học Sư phạm, 2016, tr. 94)
-• Giai đoạn từ đầu những năm 70 của thế kỉ XX đến năm 1991: Trật tự thế giới hai cực I-an-ta suy yếu và đi đến sụp đổ.
-Trật tự hai cực I-an-ta có biểu hiện suy yếu khi xu hướng hoà hoãn bắt đầu xuất hiện từ đầu những năm 70 của thế kỉ XX, với việc Liên Xô và Mỹ đạt được thoả thuận bước đầu về hạn chế vũ khí chiến lược, tiến hành cuộc gặp gỡ cấp cao đầu tiên (1972).
-EM CÓ BIẾT ?
-Chuyến thăm chính thức đầu tiên của Tổng thống Mỹ Ních-xơn tới Liên Xô diễn ra vào tháng 5 – 1972. Hai bên đã kí kết nhiều văn kiện quan trọng về hạn chế vũ khí chiến lược, về hợp tác trong các lĩnh vực: khoa học, chinh phục không gian, y học và bảo vệ môi trường,...
-15
-==End of OCR for page 3==
-==Start of OCR for page 4==
-Hình 3. Tổng thống Mỹ Ních-xơn và Tổng Bí thư Ban Chấp hành Trung ương Đảng Cộng sản Liên Xô Brê-giơ-nhép kí các văn kiện (1972)
-Từ nửa sau những năm 80 của thế kỉ XX, Liên Xô và Mỹ đẩy mạnh đối thoại, hợp tác với các cuộc gặp gỡ cấp cao. Hai nước kí kết các văn kiện hợp tác về kinh tế, thương mại, khoa học – kĩ thuật, đặc biệt là thoả thuận về việc thủ tiêu các tên lửa tầm trung ở châu Âu (1987), hạn chế cuộc chạy đua vũ trang. Năm 1989, Liên Xô và Mỹ cùng tuyên bố chấm dứt Chiến tranh lạnh.
-Sự sụp đổ của chủ nghĩa xã hội ở Đông Âu (vào cuối những năm 80 của thế kỉ XX), sự tan rã của Liên Xô (12 – 1991) đã chấm dứt sự tồn tại của Trật tự thế giới hai cực I-an-ta.
-? Khai thác thông tin và tư liệu trong mục, hãy trình bày những nét chính về quá trình tồn tại của Trật tự thế giới hai cực I-an-ta.
-2 Nguyên nhân và tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta
-a) Nguyên nhân sụp đổ
-Sự sụp đổ của Trật tự thế giới hai cực I-an-ta bắt nguồn từ nhiều nguyên nhân.
-Thứ nhất, sự đối đầu căng thẳng đã khiến cho cả hai cực Xô – Mỹ đều bị tốn kém về tài chính, suy giảm thế mạnh kinh tế, phải hạn chế cuộc chạy đua vũ trang để ổn định và củng cố vị thế của mình.
-Thứ hai, từ giữa những năm 70 của thế kỉ XX, cùng với những thay đổi trong quan hệ Xô – Mỹ là những chuyển biến theo hướng hoà dịu trong quan hệ giữa Đông Âu và Tây Âu.
-Thứ ba, sự vươn lên nhanh chóng của các nước trên thế giới nhằm thoát khỏi ảnh hưởng của hai cực, đặc biệt, thắng lợi của phong trào giải phóng dân tộc và sự ra đời của hàng loạt các quốc gia độc lập đã làm thay đổi khuôn khổ của Trật tự thế giới hai cực I-an-ta.
-Thứ tư, sự thay đổi trong cán cân kinh tế thế giới là một yếu tố góp phần làm suy yếu Trật tự thế giới hai cực I-an-ta. Sự vươn lên mạnh mẽ của Nhật Bản và các nước Tây Âu đã tạo ra những trung tâm kinh tế cạnh tranh với Mỹ; sự suy giảm sức mạnh kinh tế của Liên Xô cũng làm cho cán cân kinh tế thế giới thay đổi.
-16
-==End of OCR for page 4==
-==Start of OCR for page 5==
-Thứ năm, cuộc khủng hoảng kinh tế, xã hội và những sai lầm trong công cuộc cải tổ đã làm suy giảm sức mạnh, dẫn tới sự tan rã của Liên Xô – quốc gia đứng đầu hệ thống xã hội chủ nghĩa, cùng với đó là sự sụp đổ của Trật tự thế giới hai cực I-an-ta.
-? Nêu những nguyên nhân dẫn đến sự sụp đổ của Trật tự thế giới hai cực I-an-ta.
-b) Tác động
-Sự sụp đổ của Trật tự thế giới hai cực I-an-ta đã tác động nhiều mặt đến tình hình thế giới.
-Trước hết, sự sụp đổ của Trật tự thế giới hai cực I-an-ta đã mở ra một thời kì phát triển mới trong quan hệ quốc tế, thúc đẩy những xu hướng phát triển mới, đảm bảo lợi ích của các quốc gia, các dân tộc trong quan hệ quốc tế.
-Thứ hai, sự tan rã của Liên Xô đã làm thay đổi so sánh lực lượng với ưu thế tạm thời thuộc về Mỹ. Tuy nhiên, vai trò của các cường quốc khác, các trung tâm kinh tế, các tổ chức quốc tế, khu vực,… ngày càng gia tăng, trong khi sức mạnh của Mỹ cũng suy giảm tương đối.
-Thứ ba, sự sụp đổ của Trật tự thế giới hai cực I-an-ta dẫn đến sự hình thành một trật tự thế giới mới.
-EM CÓ BIẾT ?
-Những khoản thâm hụt ngân sách khổng lồ và nợ nước ngoài gia tăng là những thách thức lớn mà Mỹ phải đối mặt. Năm 1990, thâm hụt ngân sách của Mỹ lên đến 220 tỉ USD (gấp ba lần so với năm 1980), nợ nước ngoài tăng gần 3 000 tỉ USD. Mỹ phải cắt giảm lực lượng quân đội đồn trú ở châu Âu và một số căn cứ quân sự ở các khu vực khác trên thế giới.
-? Phân tích tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta đối với tình hình thế giới.
-LUYỆN TẬP VÀ VẬN DỤNG
-Hãy tóm tắt những nét chính về quá trình hình thành và tồn tại của Trật tự thế giới hai cực I-an-ta.
-Lập sơ đồ tư duy (theo ý tưởng của em) về nguyên nhân và tác động của sự sụp đổ Trật tự thế giới hai cực I-an-ta đối với tình hình thế giới.
-Dựa vào tư liệu sưu tầm từ sách, báo, internet và vận dụng những kiến thức đã học, hãy giải thích vì sao sự tồn tại của Trật tự thế giới hai cực I-an-ta không phù hợp với lợi ích chung của cộng đồng quốc tế.
-17
-==End of OCR for page 5==</t>
-  </si>
-  <si>
-    <t>Bài 3. Trật tự thế giới sau Chiến tranh lạnh
-Học xong bài này, em sẽ:
-◆ Nêu được xu thế phát triển chính của thế giới sau Chiến tranh lạnh.
-◆ Trình bày được khái niệm đa cực.
-◆ Nêu được xu thế đa cực trong quan hệ quốc tế sau Chiến tranh lạnh.
-◆ Vận dụng được những hiểu biết về thế giới sau Chiến tranh lạnh để giải thích những vấn đề thời sự trong quan hệ quốc tế.
-Sự kiện Bức tường Béc-lin sụp đổ (11 – 1989) là một trong những biểu tượng cho sự kết thúc của Chiến tranh lạnh. Chiến tranh lạnh kết thúc đã mở ra những xu thế phát triển mới của thế giới. Đó là những xu thế nào? Vì sao xu thế đa cực trở thành xu hướng chính trong quan hệ quốc tế sau Chiến tranh lạnh? Hãy chia sẻ những điều em biết về trật tự thế giới sau Chiến tranh lạnh.
-Hình 1. Người dân Đức trong sự kiện
-Bức tường Béc-lin sụp đổ
-1 Các xu thế phát triển chính của thế giới sau Chiến tranh lạnh
-Chiến tranh lạnh kết thúc đã mở ra một thời kì mới của thế giới với những xu thế phát triển chính: kinh tế là trọng tâm; toàn cầu hoá; đối thoại, hợp tác; đa cực trong quan hệ quốc tế,...
-• Xu thế phát triển lấy kinh tế là trọng tâm
-EM CÓ BIẾT ?
-Từ năm 1986, Việt Nam bắt đầu công cuộc Đổi mới, xây dựng nền kinh tế thị trường định hướng xã hội chủ nghĩa, được xếp trong nhóm những nền kinh tế có tốc độ tăng trưởng cao nhất thế giới, đồng thời gắn kết phát triển kinh tế với tiến bộ và công bằng xã hội.
-Sau Chiến tranh lạnh, hầu hết các quốc gia trên thế giới đều điều chỉnh chiến lược phát triển tập trung vào kinh tế, nhằm tăng cường sức mạnh, tiềm lực quốc gia, đồng thời nâng cao đời sống người dân.
-18
-==End of OCR for page 1==
-==Start of OCR for page 2==
-• Xu thế toàn cầu hoá
-Sự kết thúc của Trật tự thế giới hai cực I-an-ta và Chiến tranh lạnh, cùng với sự phát triển của cách mạng khoa học – công nghệ đã thúc đẩy mạnh mẽ quá trình toàn cầu hoá. Toàn cầu hoá là quá trình gia tăng mạnh mẽ của những mối liên hệ, sự phụ thuộc, tác động lẫn nhau giữa các quốc gia, dân tộc và khu vực trên phạm vi toàn cầu.
-• Xu thế đối thoại, hợp tác trong quan hệ quốc tế
-Nhu cầu ổn định để phát triển kinh tế, đặc biệt là xu thế toàn cầu hoá đã thúc đẩy xu thế đối thoại, cùng hợp tác, thay cho xu thế đối đầu giữa các nước có chế độ chính trị khác nhau trong quan hệ quốc tế. Xu thế đối thoại, hợp tác dựa trên cơ sở hai bên cùng có lợi, tôn trọng lẫn nhau, cùng tồn tại hoà bình đang ngày càng trở thành xu thế chủ yếu trong các mối quan hệ quốc tế.
-? Hãy nêu những xu thế phát triển chính của thế giới sau Chiến tranh lạnh.
-2 Xu thế đa cực trong quan hệ quốc tế
-a) Khái niệm đa cực
-Đa cực là một thuật ngữ trong quan hệ quốc tế dùng để chỉ một trật tự thế giới có sự tham gia của các quốc gia, các trung tâm khác nhau, trong đó không một quốc gia nào có quyền lực áp đảo đối với các quốc gia khác, cũng như chi phối sự phát triển của thế giới.
-Sự hình thành của trật tự thế giới đa cực là một tiến trình lịch sử khách quan với sự nổi lên của các cường quốc, sự gia tăng vai trò của các trung tâm, tổ chức quốc tế, phản ánh tương quan so sánh lực lượng mới trong quan hệ quốc tế sau Chiến tranh lạnh.
-? Trình bày khái niệm đa cực trong quan hệ quốc tế sau Chiến tranh lạnh.
-b) Xu thế đa cực
-Sau Chiến tranh lạnh, xu thế đa cực trở thành một trong những xu thế phát triển chính của thế giới.
-TƯ LIỆU. Nhận định về tình hình thế giới, Đại hội XII của Đảng Cộng sản Việt Nam nêu rõ: "Quá trình toàn cầu hoá và hội nhập quốc tế tiếp tục được đẩy mạnh… Cục diện thế giới theo xu hướng đa cực, đa trung tâm diễn ra nhanh hơn".
-(Đảng Cộng sản Việt Nam, Văn kiện Đại hội đại biểu toàn quốc lần thứ XII,
-NXB Chính trị quốc gia Sự thật, 2016, tr. 16)
-Biểu hiện của xu thế đa cực trước hết là sự gia tăng sức mạnh, tầm ảnh hưởng và vị thế về kinh tế, chính trị, quân sự, đối ngoại,... của các nước lớn như: Trung Quốc, Nga, Ấn Độ, Nhật Bản, một số nước thuộc Liên minh châu Âu (EU),…
-19
-==End of OCR for page 2==
-==Start of OCR for page 3==
-Hình 2. Thành phố Mum-bai – một trong những
-thành phố phát triển nhất Ấn Độ ngày nay
-EM CÓ BIẾT ?
-Mặc dù Mỹ vẫn giữ vị trí số một thế giới về kinh tế và các lĩnh vực như: vốn, khoa học – công nghệ,… nhưng vị thế của nước này đang ngày càng bị giảm dần trước sự nổi lên của các trung tâm khác. Năm 2000, GDP của Mỹ gấp khoảng 12 lần Trung Quốc, nhưng đến năm 2021 chỉ còn gấp khoảng 1,3 lần.
-EM CÓ BIẾT ?
-G20 (gồm các nước nhóm G7, EU, Ác-hen-ti-na, Ô-xtrây-li-a, Bra-xin, Trung Quốc, Mê-hi-cô, Nga, In-đô-nê-xi-a, Ấn Độ, A-rập Xê-út, Nam Phi, Hàn Quốc và Thổ Nhĩ Kỳ), chiếm 2/3 dân số thế giới, 90% GDP toàn cầu và 80% thương mại quốc tế. Được thành lập năm 1999, G20 trở thành trung tâm điều phối các nỗ lực quốc tế nhằm thúc đẩy sự phát triển kinh tế thế giới.
-Cùng với sự phát triển của Trung Quốc, Nga, thế giới còn chứng kiến sự nổi lên của Ấn Độ với mức tăng trưởng kinh tế cao liên tục trong nhiều năm. Nhật Bản và một số nước thuộc Liên minh châu Âu tiếp tục khẳng định tiềm lực kinh tế và vị thế của mình.
-Thứ hai là sự suy giảm sức mạnh tương đối của Mỹ trong tương quan so sánh với các cường quốc khác.
-Thứ ba là vai trò ngày càng gia tăng của các trung tâm, tổ chức kinh tế, tài chính quốc tế, khu vực.
-Sau Chiến tranh lạnh, các tổ chức kinh tế, tài chính khu vực, liên khu vực có vai trò ngày càng lớn đối với sự phát triển của thế giới, tiêu biểu là: Nhóm 20 nền kinh tế lớn nhất thế giới (G20); Diễn đàn Hợp tác Á – Âu (ASEM) gồm các nước thuộc Liên minh châu Âu (EU), các nước ASEAN, Trung Quốc, Nhật Bản, Hàn Quốc.
-Trong xu thế đa cực, Mỹ và Trung Quốc là hai cực có tầm ảnh hưởng lớn, nhưng các nước lớn, các trung tâm kinh tế, chính trị khác cũng đang vươn lên mạnh mẽ để khẳng định vai trò của mình trong quan hệ quốc tế.
-? Nêu những nét chính về xu thế đa cực trong quan hệ quốc tế sau Chiến tranh lạnh.
-LUYỆN TẬP VÀ VẬN DỤNG
-Lập bảng tóm tắt các xu thế phát triển chính của thế giới sau Chiến tranh lạnh.
-Bằng những kiến thức đã học và sưu tầm thêm tư liệu từ sách, báo, internet, em hãy chứng minh nhận định sau: "Hiện nay, cục diện thế giới theo xu hướng đa cực, đa trung tâm diễn ra nhanh hơn". Theo em, xu thế đó mang lại những cơ hội nào cho Việt Nam trong công cuộc phát triển đất nước?
-20
-==End of OCR for page 3==</t>
-  </si>
-  <si>
-    <t>Bài 4. Sự ra đời và phát triển  của Hiệp hội các quốc gia Đông Nam Á
-Học xong bài này, em sẽ:
-◆ Biết cách sưu tầm và sử dụng tài liệu để tìm hiểu quá trình thành lập ASEAN.
-◆ Trình bày được quá trình hình thành và mục đích thành lập của ASEAN.
-◆ Trình bày được quá trình phát triển từ ASEAN 5 đến ASEAN 10.
-◆ Nêu được các giai đoạn phát triển chính của ASEAN (từ năm 1967 đến nay).
-Trong cuốn sách Kì diệu ASEAN – Chất xúc tác cho hoà bình (The ASEAN miracle, A Catalyst for Peace), xuất bản vào dịp kỉ niệm 50 năm thành lập tổ chức ASEAN (1967 – 2017), các tác giả cho rằng thành công của ASEAN là một điều kì diệu và thế giới sẽ trở nên tốt đẹp hơn khi các khu vực đang phát triển khác noi gương sự thành công của ASEAN để tạo ra hoà bình, thịnh vượng. Vì sao ASEAN được đánh giá như một “điều kì diệu”? Hãy chia sẻ những điều em biết về sự hình thành và phát triển của ASEAN.
-Hình 1. Trang bìa cuốn sách “Kì diệu ASEAN – Chất xúc tác cho hoà bình”
-1 Quá trình hình thành và mục đích thành lập tổ chức ASEAN
-a) Quá trình hình thành tổ chức ASEAN
-ASEAN ra đời trong bối cảnh thế giới và khu vực Đông Nam Á có những chuyển biến quan trọng.
-Sau Chiến tranh thế giới thứ hai, xu hướng khu vực hoá trên thế giới bắt đầu xuất hiện và ngày càng trở nên phổ biến. Ở Đông Nam Á, các nước có nhu cầu hợp tác với nhau để cùng phát triển kinh tế, xã hội, đồng thời tạo ra sức mạnh tập thể trong việc ứng phó với sự tranh giành ảnh hưởng giữa các nước lớn đối với khu vực trong bối cảnh Chiến tranh lạnh.
-21
-==End of OCR for page 1==
-==Start of OCR for page 2==
-Đầu những năm 60 của thế kỉ XX, một số tổ chức khu vực được thành lập như: Hiệp hội Đông Nam Á (1961) gồm Ma-lai-xi-a, Phi-líp-pin và Thái Lan; Tổ chức MAPHILINDO (1963) gồm Ma-lai-xi-a, Phi-líp-pin, In-đô-nê-xi-a. Tuy nhiên, các tổ chức này chỉ tồn tại trong một thời gian ngắn, do những bất đồng trong quan hệ song phương giữa một số nước thành viên.
-Vào nửa sau những năm 60, các nước Đông Nam Á ngày càng nhận thức rõ về sự cần thiết của việc hợp tác khu vực, đồng thời quan hệ giữa các nước có những diễn biến thuận lợi cho việc thành lập một tổ chức khu vực.
-Sau các cuộc thảo luận về việc thành lập tổ chức khu vực, ngày 8 – 8 – 1967, tại Băng Cốc (Thái Lan), Ngoại trưởng năm nước: In-đô-nê-xi-a, Ma-lai-xi-a, Phi-líp-pin, Xin-ga-po và Thái Lan đã thông qua Tuyên bố ASEAN (còn gọi là Tuyên bố Băng Cốc), chính thức thành lập Hiệp hội các quốc gia Đông Nam Á (viết tắt theo tiếng Anh là ASEAN).
-Hình 2. Ngoại trưởng năm nước tham gia sáng lập ASEAN (1967)
-? Hãy trình bày quá trình hình thành tổ chức ASEAN.
-b) Mục đích thành lập ASEAN
-TƯ LIỆU. Tuyên bố ASEAN nêu rõ mục đích thành lập của ASEAN:
-Thúc đẩy sự tăng trưởng kinh tế, tiến bộ xã hội và phát triển văn hoá trong khu vực thông qua các nỗ lực chung trên tinh thần bình đẳng và hợp tác nhằm tăng cường cơ sở cho một Cộng đồng các quốc gia Đông Nam Á hoà bình và thịnh vượng.
-Thúc đẩy hoà bình và ổn định khu vực bằng việc tôn trọng công lí và nguyên tắc luật pháp trong quan hệ giữa các quốc gia trong vùng và tuân thủ các nguyên tắc của Hiến chương Liên hợp quốc.
-Thúc đẩy sự cộng tác tích cực và giúp đỡ lẫn nhau trong các vấn đề cùng quan tâm trong các lĩnh vực kinh tế, xã hội, văn hoá, khoa học – kĩ thuật và hành chính,...
-(Theo Tuyên bố ASEAN, Hiệp hội các nước Đông Nam Á (ASEAN), NXB Chính trị quốc gia, 1998, tr. 15 – 16)
-ASEAN được thành lập nhằm mục đích chính là tăng cường hợp tác kinh tế, văn hoá, xã hội, tạo điều kiện cho các nước thành viên phát triển và hội nhập với khu vực, thế giới; phấn đấu để Đông Nam Á trở thành khu vực hoà bình, tự do, thịnh vượng và ASEAN trở thành tổ chức bao gồm tất cả các quốc gia Đông Nam Á.
-? Khai thác thông tin và tư liệu trong mục, hãy trình bày mục đích thành lập ASEAN.
-22
-==End of OCR for page 2==
-==Start of OCR for page 3==
-2 Hành trình phát triển của ASEAN
-a) Từ ASEAN 5 (1967) đến ASEAN 10 (1999)
-Để thực hiện mục tiêu mở rộng thành viên bao gồm tất cả các nước trong khu vực, ASEAN đã trải qua hành trình hơn 30 năm để đưa ASEAN 5 trở thành ASEAN 10.
-1967: ASEAN 5 gồm: Thái Lan, Ma-lai-xi-a, In-đô-nê-xi-a, Xin-ga-po, Phi-líp-pin
-1984: ASEAN 6: Bru-nây gia nhập
-1995: ASEAN 7: Việt Nam gia nhập
-1997: ASEAN 9: Lào và Mi-an-ma gia nhập
-1999: ASEAN 10: Cam-pu-chia gia nhập
-Hình 3. Sơ đồ quá trình phát triển từ ASEAN 5 đến ASEAN 10
-EM CÓ BIẾT ?
-Sự kiện Việt Nam trở thành thành viên thứ bảy của ASEAN là dấu mốc quan trọng trong sự phát triển của ASEAN. Đây không chỉ là sự tăng thêm về số lượng thành viên mà còn đẩy nhanh quá trình thực hiện mục tiêu xây dựng ASEAN trở thành “ngôi nhà chung” của các quốc gia Đông Nam Á.
-Hình 4. Lễ kết nạp Vương quốc Cam-pu-chia là thành viên thứ 10 của ASEAN tại Hà Nội (Việt Nam) năm 1999
-Quá trình mở rộng ASEAN phù hợp với mong muốn, lợi ích của mỗi thành viên, đảm bảo hoà bình, ổn định của cả khu vực, đồng thời nâng cao vị thế của Hiệp hội trên trường quốc tế.
-? Trình bày quá trình phát triển từ ASEAN 5 đến ASEAN 10.
-23
-==End of OCR for page 3==
-==Start of OCR for page 4==
-b) Các giai đoạn phát triển chính của ASEAN (từ năm 1967 đến nay)
-Bảng tóm tắt các giai đoạn phát triển chính của ASEAN
-Các giai đoạn phát triển	Các tuyên bố, hiệp định quan trọng
-1967 – 1976: Giai đoạn khởi đầu, xây dựng nền móng ban đầu, tạo tiền đề cho sự hợp tác ASEAN, tập trung vào hợp tác chính trị – an ninh “xây dựng lòng tin và học cách hoà giải”.	Ra Tuyên bố về Khu vực Hoà bình, Tự do và Trung lập (ZOPFAN, 1971).
-1976 – 1999: Giai đoạn xây dựng quan hệ chính trị ổn định, tạo điều kiện phát triển và hợp tác kinh tế giữa các thành viên; mở rộng ASEAN 5 thành ASEAN 10; từng bước nâng cao uy tín ASEAN trên trường quốc tế, bước đầu mở rộng quan hệ hợp tác, đối thoại với bên ngoài.	– Ra Tuyên bố về sự Hoà hợp ASEAN (Tuyên bố Ba-li I), kí Hiệp ước Thân thiện và Hợp tác ở Đông Nam Á (TAC, 1976),...&lt;br&gt;– Kí Hiệp định khung về tăng cường hợp tác kinh tế ASEAN và thoả thuận về Khu vực Mậu dịch tự do ASEAN (AFTA, 1992), thành lập Diễn đàn khu vực ASEAN (ARF, 1994).
-1999 – 2015: Giai đoạn hoàn thiện cơ cấu tổ chức, tăng cường hợp tác nội khối và ngoại khối về chính trị – an ninh, kinh tế – thương mại và các lĩnh vực khác; khẳng định uy tín, vai trò của ASEAN.	Ra Tuyên bố Ba-li II (2003), công bố Hiến chương ASEAN (2007),...
-2015 đến nay: Thành lập và xây dựng Cộng đồng ASEAN với ba trụ cột: chính trị – an ninh, kinh tế, văn hoá – xã hội; đẩy mạnh hợp tác bên trong ASEAN và bên ngoài ASEAN với các đối tác đối thoại, nâng cao uy tín, vai trò của ASEAN ở khu vực và trên thế giới.	Ra Tuyên bố thành lập Cộng đồng ASEAN (2015), thông qua Tầm nhìn Cộng đồng ASEAN 2025 (2015), Tầm nhìn Cộng đồng ASEAN sau năm 2025 (2020),…
-? Nêu những nét chính về các giai đoạn phát triển của ASEAN từ năm 1967 đến nay.
-LUYỆN TẬP VÀ VẬN DỤNG
-Lập bảng niên biểu về quá trình mở rộng từ ASEAN 5 đến ASEAN 10.
-Có ý kiến cho rằng: Đóng góp quan trọng nhất của ASEAN trong quá trình thành lập và phát triển hơn 50 năm qua là xây dựng được môi trường hoà bình, ổn định ở Đông Nam Á. Em có đồng ý với ý kiến này không? Vì sao?
-Tìm hiểu tư liệu từ sách, báo và internet, hãy viết một bài giới thiệu ngắn gọn về các giai đoạn phát triển của ASEAN từ năm 1967 đến nay.
-24
-==End of OCR for page 4==</t>
-  </si>
-  <si>
-    <t>Bài 5. Cộng đồng ASEAN: Từ ý tưởng đến hiện thực
-Học xong bài này, em sẽ:
-◆ Biết cách sưu tầm và sử dụng tài liệu để tìm hiểu về quá trình hình thành và mục tiêu của Cộng đồng ASEAN.
-◆ Nêu được nét chính về ý tưởng, mục tiêu và kế hoạch xây dựng Cộng đồng ASEAN.
-◆ Trình bày được nội dung ba trụ cột của Cộng đồng ASEAN.
-◆ Nêu được những thách thức và triển vọng của Cộng đồng ASEAN. Có ý thức sẵn sàng tham gia vào các hoạt động xây dựng Cộng đồng ASEAN.
-Tem “Chào mừng Cộng đồng ASEAN” do các hoạ sĩ Việt Nam thiết kế, được phát hành đồng thời tại Việt Nam và các nước ASEAN vào năm 2015. Tem mang thông điệp: “Một Tầm nhìn, một Bản sắc, một Cộng đồng”. Vì sao tất cả các nước thành viên đều chào mừng Cộng đồng ASEAN? Cộng đồng ASEAN được hình thành như thế nào? Hãy chia sẻ những điều em biết về Cộng đồng ASEAN.
-Hình 1. Tem “Chào mừng Cộng đồng ASEAN” năm 2015
-1 Ý tưởng, mục tiêu và kế hoạch xây dựng Cộng đồng ASEAN
-a) Ý tưởng xây dựng Cộng đồng ASEAN
-Ý tưởng xây dựng Cộng đồng ASEAN đã khởi nguồn từ khi ASEAN thành lập. Tuyên bố Băng Cốc (1967) đã nêu ra mục tiêu xây dựng một cộng đồng thịnh vượng và hoà bình ở Đông Nam Á.
-Sau 30 năm phát triển và mở rộng, ASEAN chính thức khẳng định ý tưởng thành lập Cộng đồng ASEAN tại Hội nghị cấp cao ASEAN không chính thức được tổ chức tại Ma-lai-xi-a (1997). Các nước thành viên thông qua văn kiện Tầm nhìn ASEAN 2020, nêu rõ việc xây dựng Cộng đồng ASEAN, định hướng cho sự phát triển trong tương lai của ASEAN.
-TƯ LIỆU 1. Theo Tầm nhìn ASEAN 2020: “Toàn bộ Đông Nam Á sẽ là một cộng đồng ASEAN, nhận thức được các mối liên hệ lịch sử của mình, hiểu rõ di sản văn hoá của mình và gắn bó với nhau bằng một bản sắc chung của khu vực”.
-(Nguồn: Cổng Thông tin ASEAN – Việt Nam)
-25
-==End of OCR for page 1==
-==Start of OCR for page 2==
-Hình 2. Hội nghị cấp cao ASEAN không chính thức tại Ma-lai-xi-a (15 – 12 –1997)
-Với ý tưởng xây dựng Cộng đồng ASEAN, mục tiêu hợp tác về kinh tế, chính trị – an ninh, văn hoá – xã hội giữa các nước thành viên sẽ được phát triển lên một nấc thang mới, đáp ứng nguyện vọng của các quốc gia thành viên về một khu vực Đông Nam Á gắn kết, hữu nghị và hợp tác.
-? Khai thác thông tin và Tư liệu 1 trong mục, hãy nêu những nét chính về ý tưởng xây dựng Cộng đồng ASEAN.
-b) Mục tiêu xây dựng Cộng đồng ASEAN
-Mục tiêu xây dựng Cộng đồng ASEAN là đưa ASEAN trở thành một cộng đồng với ba trụ cột có mức độ liên kết sâu rộng hơn, ràng buộc hơn trên cơ sở pháp lí là Hiến chương ASEAN, đồng thời mở rộng hợp tác với bên ngoài.
-TƯ LIỆU 2. “Cộng đồng ASEAN sẽ được thành lập gồm ba trụ cột là hợp tác chính trị và an ninh, hợp tác kinh tế và hợp tác văn hoá – xã hội được gắn kết chặt chẽ và cùng tăng cường cho mục đích đảm bảo hoà bình, ổn định lâu dài và cùng thịnh vượng trong khu vực.”
-(Trích Tuyên bố Ba-li II (2003), Nguồn: Bộ Ngoại giao)
-? Khai thác thông tin và Tư liệu 2 trong mục, hãy nêu mục tiêu xây dựng Cộng đồng ASEAN.
-c) Kế hoạch xây dựng Cộng đồng ASEAN
-Để thực hiện mục tiêu xây dựng Cộng đồng ASEAN, các nước thành viên đã thông qua kế hoạch triển khai cụ thể trên ba trụ cột: Chính trị – An ninh, Kinh tế, Văn hoá – Xã hội.
-26
-==End of OCR for page 2==
-==Start of OCR for page 3==
-Kế hoạch được nêu rõ trong văn bản “Lộ trình xây dựng Cộng đồng ASEAN (2009 – 2015)”, được thông qua tại Hội nghị cấp cao ASEAN 14 ở Thái Lan (2009), nhằm đưa ASEAN trở thành cộng đồng gắn kết hơn về kinh tế, chính trị – an ninh, có trách nhiệm về xã hội đối với người dân.
-Về quan hệ đối ngoại, ASEAN tăng cường thực hiện các biện pháp mở rộng quan hệ hợp tác với bên ngoài, thông qua cơ chế hợp tác khu vực do ASEAN giữ vai trò chủ đạo.
-Sau sáu năm thực hiện, đến năm 2015, ASEAN đã hoàn thành về cơ bản việc triển khai các kế hoạch xây dựng cộng đồng. Trên cơ sở đó, ngày 22 – 11 – 2015, các nhà lãnh đạo ASEAN đã kí Tuyên bố thành lập Cộng đồng ASEAN, chính thức thành lập Cộng đồng ASEAN kể từ ngày 31 – 12 – 2015.
-Hình 3. Lễ kí Tuyên bố Cu-a-la Lăm-pơ thành lập Cộng đồng ASEAN (2015)
-? Trình bày những nét chính về kế hoạch xây dựng Cộng đồng ASEAN.
-2 Ba trụ cột của Cộng đồng ASEAN
-Ba trụ cột của Cộng đồng ASEAN bao gồm: Cộng đồng Chính trị – An ninh ASEAN (APSC), Cộng đồng Kinh tế ASEAN (AEC) và Cộng đồng Văn hoá – Xã hội ASEAN (ASCC).
-a) Cộng đồng Chính trị – An ninh ASEAN (APSC)
-Cộng đồng Chính trị – An ninh ASEAN được xây dựng trên nền tảng những thành quả hợp tác chính trị – an ninh đã đạt được, nhằm mục tiêu tạo dựng môi trường hoà bình và an ninh ở khu vực, nâng hợp tác chính trị – an ninh lên một nấc thang mới cao hơn và chặt chẽ hơn, trên cơ sở các nguyên tắc cơ bản của ASEAN.
-TƯ LIỆU 3. Kế hoạch Tổng thể xây dựng Cộng đồng Chính trị – An ninh ASEAN (2009 – 2015) bao gồm ba nội dung chính: “Xây dựng một cộng đồng dựa trên các giá trị và chuẩn mực chung; Tạo dựng một khu vực gắn kết, hoà bình và tự cường với trách nhiệm chung đối với an ninh toàn diện; Hướng tới một khu vực năng động và rộng mở với bên ngoài trong một thế giới ngày càng liên kết và tuỳ thuộc”.
-(Nguồn: Cổng Thông tin ASEAN – Việt Nam)
-? Khai thác thông tin và Tư liệu 3 trong mục, hãy trình bày nội dung chính của Cộng đồng Chính trị – An ninh ASEAN.
-27
-==End of OCR for page 3==
-==Start of OCR for page 4==
-b) Cộng đồng Kinh tế ASEAN (AEC)
-Cộng đồng Kinh tế ASEAN là sự tiếp nối các chương trình hợp tác kinh tế của ASEAN trước đây, được mở rộng hơn về phạm vi, mức độ hợp tác kinh tế, thương mại,...
-Hình 4. Các đại biểu tham dự Hội nghị Hội đồng Kinh tế ASEAN lần thứ 18 tại Thái Lan (2019)
-EM CÓ BIẾT ?
-Sau khi AEC thành lập, hợp tác kinh tế giữa các nước ASEAN gia tăng nhanh chóng. Thương mại giữa Việt Nam – ASEAN tăng từ hơn 41 tỉ USD (2016) lên hơn 70 tỉ USD (2021).
-Nội dung chính của Cộng đồng Kinh tế ASEAN bao gồm: tạo ra một thị trường và cơ sở sản xuất chung, trong đó có sự lưu chuyển tự do của hàng hoá, dịch vụ, đầu tư, vốn và lao động có tay nghề; xây dựng khu vực kinh tế có sức cạnh tranh cao, năng động, phát triển đồng đều, hội nhập đầy đủ vào nền kinh tế toàn cầu.
-? Hãy trình bày nội dung chính của Cộng đồng Kinh tế ASEAN.
-c) Cộng đồng Văn hoá – Xã hội ASEAN (ASCC)
-Cộng đồng Văn hoá – Xã hội ASEAN là một khuôn khổ hợp tác chặt chẽ với các quy định và tiêu chuẩn chung để tạo sự hài hoà, bình đẳng và công bằng xã hội, nâng cao ý thức về cộng đồng và bản sắc chung ASEAN.
-TƯ LIỆU 4. Kế hoạch Tổng thể xây dựng Cộng đồng Văn hoá – Xã hội ASEAN (2009) xác định sáu nội dung chính bao gồm: Phát triển con người; Phúc lợi và bảo hiểm xã hội; Bình đẳng xã hội và các quyền; Bảo đảm bền vững về môi trường; Xây dựng bản sắc ASEAN; Thu hẹp khoảng cách phát triển.
-(Theo Bộ Công Thương, Cộng đồng Kinh tế ASEAN 2015, NXB Thế giới, 2016, tr. 10)
-28
-==End of OCR for page 4==
-==Start of OCR for page 5==
-Có nền tảng từ sự phát triển các giá trị văn hoá truyền thống lâu đời, Cộng đồng Văn hoá – Xã hội ASEAN là một trụ cột quan trọng, gắn kết và tạo thuận lợi cho việc xây dựng hai trụ cột Kinh tế và Chính trị – An ninh.
-? Khai thác thông tin và Tư liệu 4 trong mục, hãy trình bày nội dung chính của Cộng đồng Văn hoá – Xã hội ASEAN.
-3 Cộng đồng ASEAN sau năm 2015
-• Tầm nhìn ASEAN sau năm 2015
-Sau khi thành lập Cộng đồng ASEAN, các nước ASEAN tiếp tục đưa ra định hướng cho một giai đoạn phát triển mới sau năm 2015 với nội dung định hướng là tiếp tục củng cố, làm sâu sắc hơn các lĩnh vực hợp tác.
-Hội nghị Cấp cao ASEAN lần thứ 37 tại Hà Nội (2020) đã nhất trí thông qua việc xây dựng Tầm nhìn Cộng đồng ASEAN sau năm 2025, hướng tới việc gắn kết chặt chẽ các nội dung hợp tác trên cả ba trụ cột (Cộng đồng Chính trị – An ninh, Cộng đồng Kinh tế và Cộng đồng Văn hoá – Xã hội), đồng thời bổ sung những nội dung mới như: hợp tác về chuyển đổi số, phát triển nền kinh tế số, kinh tế xanh,...
-Hình 5. Tổng Bí thư, Chủ tịch nước Nguyễn Phú Trọng phát biểu chào mừng khai mạc Hội nghị cấp cao ASEAN lần thứ 37 (2020)
-• Những thách thức và triển vọng của Cộng đồng ASEAN
-Trong quá trình phát triển, Cộng đồng ASEAN phải đối mặt với những thách thức trong nội khối và từ bên ngoài.
-Trong nội khối, những thách thức cơ bản đối với Cộng đồng ASEAN về chính trị là sự đa dạng về chế độ chính trị, tình hình chính trị ở một số nước còn phức tạp, còn tồn tại một số mâu thuẫn trong quan hệ song phương,... Về kinh tế, sự chênh lệch về thu nhập, trình độ phát triển,... giữa các nước gây khó khăn trong hợp tác nội khối; sự tương đồng trong sản xuất một số ngành nghề cũng tạo ra sự cạnh tranh trong xuất khẩu,…
-29
-==End of OCR for page 5==
-==Start of OCR for page 6==
-Bên cạnh đó, những thách thức từ bên ngoài cũng tác động đến Cộng đồng ASEAN như: cạnh tranh ảnh hưởng của các nước lớn đối với khu vực, diễn biến phức tạp của tình hình Biển Đông và tình hình quốc tế; biến đổi khí hậu, ô nhiễm môi trường, dịch bệnh,... Để vượt qua những thách thức, các nước ASEAN đã và đang đẩy nhanh quá trình triển khai các kế hoạch đã đề ra vì lợi ích chung, lâu dài của cả cộng đồng.
-EM CÓ BIẾT ?
-Năm 2021, ASEAN là nền kinh tế lớn thứ năm thế giới với GDP khoảng 3 300 tỉ USD, dự báo đến năm 2030 sẽ trở thành nền kinh tế thứ tư thế giới.
-Về triển vọng, ASEAN sẽ tiếp tục phát triển với mức độ liên kết, hợp tác ngày càng sâu rộng trên cả ba trụ cột, tiếp tục là một trong những khu vực phát triển năng động nhất trên thế giới. Về đối ngoại, ASEAN có quan hệ rộng mở với các đối tác bên ngoài, đồng thời có uy tín, vị thế ngày càng cao trong khu vực và trên thế giới.
-? Nêu những thách thức và triển vọng của Cộng đồng ASEAN.
-LUYỆN TẬP VÀ VẬN DỤNG
-Tóm tắt nét chính về ý tưởng, mục tiêu và kế hoạch xây dựng Cộng đồng ASEAN.
-Lập bảng thống kê (theo gợi ý dưới đây vào vở) về nội dung ba trụ cột của Cộng đồng ASEAN.
-Cộng đồng Chính trị – An ninh	Cộng đồng Kinh tế	Cộng đồng Văn hoá – Xã hội
-?	?	?
-Sưu tầm tư liệu từ sách, báo, internet và vận dụng kiến thức đã học, hãy viết một bài giới thiệu ngắn về những hoạt động của em để góp phần xây dựng Cộng đồng ASEAN vững mạnh, phát triển.
-30
-==End of OCR for page 6==</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1185,8 +1258,21 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1205,8 +1291,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DAF8"/>
+        <bgColor rgb="FFC9DAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor rgb="FFC9DAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1284,15 +1388,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -1367,85 +1462,85 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1785,7 +1880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:O28"/>
+  <dimension ref="B1:P28"/>
   <sheetFormatPr defaultRowHeight="36.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -1802,43 +1897,48 @@
     <col min="12" max="12" width="15.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="33" style="2" customWidth="1"/>
-    <col min="15" max="15" width="8" customWidth="1"/>
+    <col min="15" max="15" width="53.28515625" customWidth="1"/>
+    <col min="16" max="16" width="43.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="31" t="s">
+    <row r="1" spans="2:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25" t="s">
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25" t="s">
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-    </row>
-    <row r="2" spans="2:15" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="32"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="27"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="P1" s="28"/>
+    </row>
+    <row r="2" spans="2:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="24"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="22"/>
       <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1866,16 +1966,18 @@
       <c r="N2" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="2:15" ht="119.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="44">
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
+    </row>
+    <row r="3" spans="2:16" ht="119.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="35">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="32" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>46</v>
@@ -1893,13 +1995,18 @@
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
-      <c r="O3" s="36"/>
-    </row>
-    <row r="4" spans="2:15" ht="152.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="45"/>
-      <c r="C4" s="42"/>
+      <c r="O3" s="44" t="s">
+        <v>70</v>
+      </c>
+      <c r="P3" s="44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16" ht="152.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="36"/>
+      <c r="C4" s="33"/>
       <c r="D4" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>47</v>
@@ -1917,13 +2024,18 @@
       <c r="L4" s="8"/>
       <c r="M4" s="8"/>
       <c r="N4" s="8"/>
-      <c r="O4" s="36"/>
-    </row>
-    <row r="5" spans="2:15" ht="95.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="45"/>
-      <c r="C5" s="42"/>
+      <c r="O4" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="P4" s="44" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" ht="95.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="36"/>
+      <c r="C5" s="33"/>
       <c r="D5" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>48</v>
@@ -1943,13 +2055,16 @@
       <c r="L5" s="8"/>
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
-      <c r="O5" s="36"/>
-    </row>
-    <row r="6" spans="2:15" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45"/>
-      <c r="C6" s="42"/>
+      <c r="O5" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="P5" s="44"/>
+    </row>
+    <row r="6" spans="2:16" ht="168" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="36"/>
+      <c r="C6" s="33"/>
       <c r="D6" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>49</v>
@@ -1969,13 +2084,18 @@
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
-      <c r="O6" s="36"/>
-    </row>
-    <row r="7" spans="2:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="46"/>
-      <c r="C7" s="43"/>
+      <c r="O6" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="P6" s="44" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="37"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>50</v>
@@ -1993,17 +2113,18 @@
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
-      <c r="O7" s="36"/>
-    </row>
-    <row r="8" spans="2:15" ht="172.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="44">
+      <c r="O7" s="44"/>
+      <c r="P7" s="44"/>
+    </row>
+    <row r="8" spans="2:16" ht="172.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="35">
         <v>2</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>51</v>
@@ -2023,13 +2144,18 @@
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
-      <c r="O8" s="36"/>
-    </row>
-    <row r="9" spans="2:15" ht="246" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="45"/>
-      <c r="C9" s="42"/>
+      <c r="O8" s="44" t="s">
+        <v>77</v>
+      </c>
+      <c r="P8" s="44" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="246" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="36"/>
+      <c r="C9" s="33"/>
       <c r="D9" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>52</v>
@@ -2049,13 +2175,16 @@
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
-      <c r="O9" s="36"/>
-    </row>
-    <row r="10" spans="2:15" ht="221.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="45"/>
-      <c r="C10" s="42"/>
+      <c r="O9" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="P9" s="44"/>
+    </row>
+    <row r="10" spans="2:16" ht="221.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="36"/>
+      <c r="C10" s="33"/>
       <c r="D10" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>53</v>
@@ -2075,13 +2204,16 @@
       <c r="L10" s="8"/>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
-      <c r="O10" s="36"/>
-    </row>
-    <row r="11" spans="2:15" ht="251.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="45"/>
-      <c r="C11" s="42"/>
+      <c r="O10" s="45" t="s">
+        <v>82</v>
+      </c>
+      <c r="P10" s="44"/>
+    </row>
+    <row r="11" spans="2:16" ht="251.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="36"/>
+      <c r="C11" s="33"/>
       <c r="D11" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>54</v>
@@ -2101,13 +2233,16 @@
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
-      <c r="O11" s="36"/>
-    </row>
-    <row r="12" spans="2:15" ht="122.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="46"/>
-      <c r="C12" s="43"/>
+      <c r="O11" s="44" t="s">
+        <v>80</v>
+      </c>
+      <c r="P11" s="44"/>
+    </row>
+    <row r="12" spans="2:16" ht="122.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="37"/>
+      <c r="C12" s="34"/>
       <c r="D12" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>61</v>
@@ -2123,17 +2258,18 @@
       <c r="L12" s="8"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
-      <c r="O12" s="36"/>
-    </row>
-    <row r="13" spans="2:15" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="44">
+      <c r="O12" s="44"/>
+      <c r="P12" s="44"/>
+    </row>
+    <row r="13" spans="2:16" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="35">
         <v>3</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>55</v>
@@ -2151,13 +2287,14 @@
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
-      <c r="O13" s="36"/>
-    </row>
-    <row r="14" spans="2:15" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="45"/>
-      <c r="C14" s="42"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+    </row>
+    <row r="14" spans="2:16" ht="86.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="36"/>
+      <c r="C14" s="33"/>
       <c r="D14" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>56</v>
@@ -2173,13 +2310,14 @@
       <c r="L14" s="8"/>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
-      <c r="O14" s="36"/>
-    </row>
-    <row r="15" spans="2:15" ht="107.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="45"/>
-      <c r="C15" s="42"/>
+      <c r="O14" s="44"/>
+      <c r="P14" s="44"/>
+    </row>
+    <row r="15" spans="2:16" ht="107.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="36"/>
+      <c r="C15" s="33"/>
       <c r="D15" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>57</v>
@@ -2197,13 +2335,14 @@
       <c r="L15" s="8"/>
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
-      <c r="O15" s="36"/>
-    </row>
-    <row r="16" spans="2:15" ht="107.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="45"/>
-      <c r="C16" s="42"/>
+      <c r="O15" s="44"/>
+      <c r="P15" s="44"/>
+    </row>
+    <row r="16" spans="2:16" ht="107.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="36"/>
+      <c r="C16" s="33"/>
       <c r="D16" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>58</v>
@@ -2221,13 +2360,14 @@
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
-      <c r="O16" s="36"/>
-    </row>
-    <row r="17" spans="2:15" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="46"/>
-      <c r="C17" s="43"/>
+      <c r="O16" s="44"/>
+      <c r="P16" s="44"/>
+    </row>
+    <row r="17" spans="2:16" ht="91.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="37"/>
+      <c r="C17" s="34"/>
       <c r="D17" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>59</v>
@@ -2243,9 +2383,10 @@
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
-      <c r="O17" s="36"/>
-    </row>
-    <row r="18" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O17" s="44"/>
+      <c r="P17" s="44"/>
+    </row>
+    <row r="18" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="12">
         <v>4</v>
       </c>
@@ -2261,9 +2402,10 @@
       <c r="L18" s="8"/>
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
-      <c r="O18" s="36"/>
-    </row>
-    <row r="19" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O18" s="41"/>
+      <c r="P18" s="41"/>
+    </row>
+    <row r="19" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="12">
         <v>5</v>
       </c>
@@ -2279,9 +2421,10 @@
       <c r="L19" s="8"/>
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
-      <c r="O19" s="36"/>
-    </row>
-    <row r="20" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O19" s="41"/>
+      <c r="P19" s="41"/>
+    </row>
+    <row r="20" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="12">
         <v>6</v>
       </c>
@@ -2297,9 +2440,10 @@
       <c r="L20" s="8"/>
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
-      <c r="O20" s="36"/>
-    </row>
-    <row r="21" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O20" s="41"/>
+      <c r="P20" s="41"/>
+    </row>
+    <row r="21" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="12">
         <v>7</v>
       </c>
@@ -2315,9 +2459,10 @@
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
-      <c r="O21" s="36"/>
-    </row>
-    <row r="22" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O21" s="41"/>
+      <c r="P21" s="41"/>
+    </row>
+    <row r="22" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="12">
         <v>8</v>
       </c>
@@ -2333,9 +2478,10 @@
       <c r="L22" s="8"/>
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
-      <c r="O22" s="36"/>
-    </row>
-    <row r="23" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O22" s="42"/>
+      <c r="P22" s="43"/>
+    </row>
+    <row r="23" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="12">
         <v>9</v>
       </c>
@@ -2351,9 +2497,10 @@
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
-      <c r="O23" s="36"/>
-    </row>
-    <row r="24" spans="2:15" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O23" s="42"/>
+      <c r="P23" s="43"/>
+    </row>
+    <row r="24" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="12">
         <v>10</v>
       </c>
@@ -2369,17 +2516,18 @@
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
-      <c r="O24" s="36"/>
-    </row>
-    <row r="25" spans="2:15" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="37" t="s">
+      <c r="O24" s="42"/>
+      <c r="P24" s="43"/>
+    </row>
+    <row r="25" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="28" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="17"/>
-      <c r="E25" s="18"/>
+      <c r="E25" s="17"/>
       <c r="F25" s="4">
         <v>12</v>
       </c>
@@ -2410,108 +2558,121 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="2:15" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="37"/>
-      <c r="C26" s="19" t="s">
+      <c r="O25" s="46"/>
+      <c r="P25" s="46"/>
+    </row>
+    <row r="26" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="28"/>
+      <c r="C26" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="19"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="21">
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="19">
         <f>(F25/40)*100</f>
         <v>30</v>
       </c>
-      <c r="G26" s="21">
+      <c r="G26" s="19">
         <f>(G25/40)*100</f>
         <v>20</v>
       </c>
-      <c r="H26" s="21">
+      <c r="H26" s="19">
         <f t="shared" ref="H26:N26" si="1">(H25/40)*100</f>
         <v>10</v>
       </c>
-      <c r="I26" s="21">
+      <c r="I26" s="19">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="J26" s="21">
+      <c r="J26" s="19">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="K26" s="21">
+      <c r="K26" s="19">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L26" s="21">
+      <c r="L26" s="19">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="M26" s="21">
+      <c r="M26" s="19">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N26" s="21">
+      <c r="N26" s="19">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="2:15" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="37"/>
-      <c r="C27" s="19" t="s">
+      <c r="O26" s="46"/>
+      <c r="P26" s="46"/>
+    </row>
+    <row r="27" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="28"/>
+      <c r="C27" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="38">
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="29">
         <v>24</v>
       </c>
-      <c r="G27" s="39"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="38">
+      <c r="G27" s="30"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="29">
         <f>I25+J25+K25</f>
         <v>16</v>
       </c>
-      <c r="J27" s="39"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="38">
+      <c r="J27" s="30"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="29">
         <f>L25+M25+N25</f>
         <v>0</v>
       </c>
-      <c r="M27" s="39"/>
-      <c r="N27" s="40"/>
-    </row>
-    <row r="28" spans="2:15" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="37"/>
-      <c r="C28" s="19" t="s">
+      <c r="M27" s="30"/>
+      <c r="N27" s="31"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="46"/>
+    </row>
+    <row r="28" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="28"/>
+      <c r="C28" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="33">
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="25">
         <f>(F27/40)*100</f>
         <v>60</v>
       </c>
-      <c r="G28" s="34"/>
-      <c r="H28" s="35"/>
-      <c r="I28" s="33">
+      <c r="G28" s="26"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="25">
         <f>(I27/40)*100</f>
         <v>40</v>
       </c>
-      <c r="J28" s="34"/>
-      <c r="K28" s="35"/>
-      <c r="L28" s="33">
+      <c r="J28" s="26"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="25">
         <f>(L27/40)*100</f>
         <v>0</v>
       </c>
-      <c r="M28" s="34"/>
-      <c r="N28" s="35"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="O1:P2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="L28:N28"/>
-    <mergeCell ref="O3:O24"/>
     <mergeCell ref="B25:B28"/>
     <mergeCell ref="F27:H27"/>
     <mergeCell ref="I27:K27"/>
@@ -2524,11 +2685,6 @@
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="B13:B17"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update: prompt & schema
</commit_message>
<xml_diff>
--- a/data/input/07. SỬ 12. ma trận KSCL lần 1 (1).xlsx
+++ b/data/input/07. SỬ 12. ma trận KSCL lần 1 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\App\matrixquesgen\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274D177D-48D4-4E35-B827-7E93361FAAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52160665-B1A3-49D9-A6B9-4057695F4E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="76">
   <si>
     <t>Stt</t>
   </si>
@@ -999,77 +999,7 @@
 ==End of OCR for page 6==</t>
   </si>
   <si>
-    <t>**“Hậu quả tàn khốc của Chiến tranh thế giới thứ hai đã thôi thúc các nước Đồng minh nhất trí về nguyên tắc cần phải thành lập một cơ chế mới, một tổ chức quốc tế mới hoạt động hiệu quả hơn so với Hội Quốc liên(1) để đảm nhận sứ mệnh cao cả gìn giữ hòa bình và ngăn ngừa một cuộc chiến tranh thế giới.... Quyết tâm này được thể hiện rất rõ tại Tuyên bố ở Hội nghị Mát-xcơ-va (tháng 10-1943) và ở Hội nghị Tê-hê-ran (tháng 12-1943) giữa Liên Xô, Anh, Hoa Kỳ và Trung Quốc.... Sau hàng loạt trao đổi trong các năm 1943 - 1944, ngày 25-4-1945, đại biểu của 50 quốc gia đã họp tại Xan Phran-xi-xcô (Hoa Kỳ), soạn thảo và thống nhất thông qua Bản Hiến chương Liên hợp quốc gồm 111 điều vào ngày 25-6-1945.... Ngày 24-10-1945 đánh dấu lịch sử của Liên hợp quốc khi bản Hiến chương được 5 nước thành viên Hội đồng Bảo an cùng hầu hết các quốc gia tham gia ký kết đã phê chuẩn và có hiệu lực.”**  
-(“Liên hợp quốc 70 năm hình thành và phát triển”, Tạp chí Cộng sản, https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/35552/lien-hop-quoc-70-nam-hinh-thanh-va-phat-tr...)[1][3]
-[1](https://tapchicongsan.org.vn)
-[2](https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/to-chuc-quoc-te/lien-hop-quoc-un-3283)
-[3](https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/35552/lien-hop-quoc-70-nam-hinh-thanh-va-phat-trien.aspx)
-[4](https://hcmcpv.org.vn/tin-tuc/viet-nam-va-su-no-luc-khang-dinh-vi-the-trong-to-chuc-lien-hop-quoc-1491884544)
-[5](https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/7754/thong-tin-co-ban-ve-lien-hop-quoc.aspx)
-[6](https://www.tapchicongsan.org.vn/media-story/-/asset_publisher/V8hhp4dK31Gf/content/quan-he-viet-nam-lien-hop-quoc-khoi-dau-hop-tac-moi-vi-mot-tuong-lai-tot-dep-cua-nhan-loai)
-[7](https://www.tapchicongsan.org.vn/the-gioi-van-de-su-kien/-/2018/2946/lien-hop-quoc-trong-boi-canh-quoc-te-moi.aspx)
-[8](https://tapchicongsan.org.vn/web/guest/quoc-phong-an-ninh-oi-ngoai1/-/2018/47141/viet-nam-gia-nhap-lien-hop-quoc--moc-son-lich-su.aspx)
-[9](https://ttdn.vn/nghien-cuu-trao-doi/su-kien-binh-luan/hanh-trinh-80-nam-lien-hop-quoc-tu-qua-khu-den-tuong-lai-113810)
-[10](https://www.studocu.vn/vn/document/hoc-vien-bao-chi-va-tuyen-truyen/quan-he-quoc-te/lien-hop-quoc-doc-mon-quan-he-quoc-te-lien-hop-quoc/61873952)
-[11](https://tapchicongsan.org.vn/web/guest/quoc-phong-an-ninh-oi-ngoai1/-/2018/47741/lien-hop-quoc-va-nhung-dong-gop-cua-viet-nam.aspx)</t>
-  </si>
-  <si>
-    <t>Điều 1 của Hiến chương nêu rõ bốn (04) mục tiêu cơ bản của Liên Hợp quốc là: (1) Duy trì hoà bình và an ninh quốc tế; (2) Thúc đẩy quan hệ hữu nghị giữa các quốc gia trên cơ sở tôn trọng nguyên tắc bình đẳng về quyền lợi giữa các dân tộc và nguyên tắc dân tộc tự quyết; (3) Thực hiện hợp tác quốc tế thông qua giải quyết các vấn đề quốc tế trên các lĩnh vực kinh tế, xã hội, văn hoá và nhân đạo trên cơ sở tôn trọng các quyền con người và quyền tự do cơ bản cho tất cả mọi người, không phân biệt chủng tộc, màu da, ngôn ngữ và tôn giáo; (4) Xây dựng Liên Hợp quốc làm trung tâm điều hoà các nỗ lực quốc tế vì các mục tiêu chung. Và 6 nguyên tắc hoạt động chủ yếu của Liên Hợp quốc là: (1) Bình đẳng về chủ quyền quốc gia; (2) Tôn trọng toàn vẹn lãnh thổ và độc lập chính trị quốc gia; (3) Cấm đe doạ sử dụng vũ lực hoặc sử dụng vũ lực trong quan hệ quốc tế; (4) Không can thiệp vào công việc nội bộ các nước; (5) Tôn trọng các nghĩa vụ quốc tế và luật pháp quốc tế; và (6) Giải quyết các tranh chấp quốc tế bằng biện pháp hoà bình.”
-(“Thông tin cơ bản về Liên hợp quốc”, Tạp chí Cộng sản, https://tapchicongsan.org.vn/web/guest/hoat-ong-cua-lanh-ao-ang-nha-nuoc/-/2018/7754/thong-tin-co-ban-ve-lien-hop-quoc.aspx)[1]</t>
-  </si>
-  <si>
-    <t>Chiến tranh thế giới thứ II kết thúc, phe Trục phát xít Đức - Italia - Nhật Bản thất bại hoàn toàn, Liên Xô và các nước Đồng minh giành thắng lợi. Cuộc chiến này đã làm thay đổi căn bản tương quan sức mạnh giữa các nước, trung tâm quyền lực trong quan hệ quốc tế, đưa đến hình thành một trật tự thế giới mới cả về chính trị và kinh tế.
-Hội nghị nguyên thủ ba nước là Anh, Mỹ và Liên Xô tại Teheran (tháng 10 - 1943), đặc biệt các cuộc đàm phán tại Yalta (tháng 2 - 1945) và Posdam (tháng 7-8 năm 1945) đã sắp xếp lại quyền lực trong quan hệ quốc tế và từ đây thế giới hình thành nên hệ thống hay trật tự thế giới hai cực, một cực do Liên Xô đứng đầu và cực kia do Mỹ đứng đầu đối nghịch nhau về ý thức hệ chính trị - tư tưởng, kinh tế và quân sự.</t>
-  </si>
-  <si>
-    <t>Trong thời kỳ này, mặc dù nước Anh trong hai phần đầu của thế kỷ XIX, nước Mỹ từ đầu thế kỷ XX có sức mạnh vượt trội, nhưng không thể thiết lập được một thế giới đơn cực bởi sự nổi lên của các cường quốc mới như Pháp, Đức, Nhật và nhất là Liên Xô sau đó. Trật tự thế giới hai cực được hình thành sau Hội nghị Yalta năm 1945 và kết thúc vào năm 1991. Đặc trưng của giai đoạn này là siêu cường Liên Xô và Mỹ đối đầu nhau về ý thức và quân sự. Thế giới bị phân chia thành hai phe, phe XHCN do Liên Xô dẫn dắt và phe TBCN do Mỹ đứng đầu. Hầu hết các quan hệ quốc tế  bị chi phối bởi tư duy của Chiến tranh Lạnh, cho dù hệ thống hay trật tự quốc tế dựa trên luật lệ đã được hình thành, điển hình là hệ thống Liên hợp quốc. Còn trật tự thế giới đơn cực hay khoảnh khắc của trật tự đơn cực do Mỹ nắm vai trò chủ đạo được thiết lập từ khi Liên Xô tan rã đến cuối thập niên đầu thế kỷ XXI.</t>
-  </si>
-  <si>
-    <t>“Chiến tranh lạnh kết thúc, thế giới chuyển từ thời đại địa chính trị sang thời đại của địa kinh tế, mà ở đó cuộc đua tranh giữa các quốc gia dù vẫn được xác định bởi ‘logic của xung đột’ nhưng thông qua ‘ngôn ngữ thương mại’. Theo quan điểm của Luttwak, địa kinh tế là hình thức mới của sự cạnh tranh sức mạnh giữa các quốc gia sau chiến tranh lạnh. Ông cho rằng, chính trị quốc tế thời kỳ hậu chiến tranh lạnh mặc dù vẫn bị chi phối bởi cạnh tranh sức mạnh giữa các nhà nước nhưng chiến trường chủ yếu là kinh tế thay vì quân sự, phương tiện ưa thích được các nhà nước sử dụng để theo đuổi các mục tiêu đối kháng nhau sẽ là kinh tế hơn là quân sự.” (“Mối quan hệ giữa địa chính trị và địa kinh tế - Lý luận và thực tiễn”, Tạp chí Lý luận chính trị, 26/09/2019, https://lyluanchinhtri.vn/moi-quan-he-giua-dia-chinh-tri-va-dia-kinh-te-ly-luan-va-thuc-tien-431.html”)</t>
-  </si>
-  <si>
-    <t>Trong khi đó, sau Chiến tranh Thế giới thứ II, các trào lưu hình thành “chủ nghĩa khu vực” trên thế giới đã xuất hiện và cùng với nó là sự ra đời của Cộng đồng Kinh tế Châu Âu (EEC); Khu vực Thương mại Tự do Mỹ Latin (LAFTA); Thị trường chung Trung Mỹ (CACM)....Việc thành lập các tổ chức khu vực này đã tác động đến việc hình thành ASEAN.
-Từ kinh nghiệm của EEC, các nước Đông Nam Á đều thấy rằng việc hình thành các tổ chức khu vực sẽ giúp thúc đẩy sự tăng trưởng kinh tế thông qua tăng cường hợp tác kinh tế, buôn bán và phân công lao động.
-Về mặt chính trị, các tổ chức khu vực giúp củng cố tình đoàn kết khu vực và giúp các nước vừa và nhỏ có tiếng nói mạnh mẽ hơn trong các vấn đề quốc tế. Còn về mặt xã hội, chủ nghĩa khu vực có thể đưa ra các phương hướng hợp tác để giải quyết có hiệu quả các vấn đề đặt ra cho các nước thành viên.
-Sau nhiều cuộc thảo luận, ngày 8/8/1967, Bộ trưởng Ngoại giao các nước Indonesia, Thái Lan, Philippines, Singapore và Phó Thủ tướng Malaysia ký tại Bangkok bản Tuyên bố thành lập Hiệp hội các quốc gia Đông Nam Á (ASEAN).
-Từ 5 nước thành viên ban đầu, đến nay ASEAN đã có 10 quốc gia thành viên, gồm Indonesia, Thái Lan, Philippines, Singapore, Malaysia, Bruney (năm 1984), Việt Nam (năm1995), Lào (năm 1997), Myanmar (năm 1997) và Campuchia (năm1999).
-ASEAN có diện tích 4,5 triệu km2, dân số khoảng 575 triệu người và tổng sản phẩm quốc nội (GDP) đạt 2.487 tỷ USD (ước tính năm 2009).
-Thực tiễn đã chứng minh rằng, một Đông Nam Á thống nhất đã thúc đẩy cho hợp tác và vị thế ASEAN ngày càng lớn mạnh, là tiền đề quan trọng để ASEAN trở thành một cộng đồng.</t>
-  </si>
-  <si>
-    <t>Những cột mốc phát triển quan trọng
-+ Tuyên bố ASEAN:
-Ngày 8/8/1967, tại Bangkok, Thái Lan, Bộ trưởng phụ trách các vấn đề chính trị kiêm Bộ trưởng Ngoại giao Indonesia, Phó Thủ tướng Malaysia, Bộ trưởng Ngoại giao Philippines, Bộ trưởng Ngoại giao Singapore và Bộ trưởng Ngoại giao Thái Lan đã ra Tuyên bố ASEAN.
-Đây là Tuyên bố thành lập Hiệp hội các quốc gia Đông Nam Á với mục tiêu đẩy mạnh tăng trưởng kinh tế, tiến bộ xã hội, phát triển văn hóa; tăng cường hợp tác, giúp đỡ lẫn nhau cũng như thúc đẩy hòa bình, ổn định trong khu vực.
-+ Tuyên bố về khu vực hòa bình, tự do và trung lập:
-Ngày 27/11/1971, tại Kuala Lumpur, Malaysia, Bộ trưởng Ngoại giao Indonesia, Malaysia, Philippines, Xingapo và Đặc phái viên của Hội đồng Hành pháp Quốc gia Thái Lan đã ký và công bố “Tuyên bố về khu vực hòa bình, tự do và trung lập ở Đông Nam Á”- Tuyên bố ZOPFAN.
-Tuyên bố quan trọng này đã định ra các mục tiêu cơ bản và lâu dài của ASEAN là xây dựng Đông Nam á thành một khu vực hòa bình, tự do và trung lập, không có sự can thiệp dưới bất cứ hình thức nào của các cường quốc bên ngoài.
-+ Hiệp ước Thân thiện và Hợp tác Đông Nam Á:
-Ngày 24/2/1976, tại Bali, Indonesia, nguyên thủ quốc gia các nước ASEAN ký Hiệp ước Thân thiện và Hợp tác ở Đông Nam Á (Hiệp ước Bali).Hiệp ước nhằm thúc đẩy hòa bình vĩnh viễn, tình hữu nghị và hợp tác lâu bền giữa nhân dân các bên tham gia Hiệp ước, góp phần tăng cường sức mạnh, tình đoàn kết và quan hệ chặt chẽ hơn giữa các nước Đông Nam Á.</t>
-  </si>
-  <si>
-    <t>Ngay sau khi chiến tranh chấm dứt, các tổ chức phát triển của Liên hợp quốc đã nhanh chóng hỗ trợ Việt Nam khắc phục hậu quả chiến tranh, tái thiết đất nước và vượt qua những khó khăn kinh tế - xã hội hết sức nặng nề. Liên hợp quốc là cầu nối để Việt Nam tiếp cận nguồn viện trợ nước ngoài và từng bước phá vỡ thế bao vây, cấm vận. Trong giai đoạn đổi mới, Liên hợp quốc tiếp tục hỗ trợ Việt Nam phát triển nguồn lực khoa học - kỹ thuật, nâng cao năng lực, hoàn thiện khuôn khổ pháp luật, chính sách, xóa đói, giảm nghèo. Nguồn vốn, tri thức, kinh nghiệm từ hệ thống Liên hợp quốc không chỉ góp phần giúp Việt Nam thúc đẩy công nghiệp hóa, hiện đại hóa đất nước, đạt nhiều thành tựu phát triển kinh tế - xã hội và thực hiện các mục tiêu phát triển toàn cầu, mà còn đóng vai trò quan trọng trong tiến trình hội nhập quốc tế của Việt Nam. 
-Về phía mình, Việt Nam không ngừng khẳng định vai trò chủ động và đóng góp tích cực vào các hoạt động của Liên hợp quốc, chia sẻ sâu sắc những giá trị cốt lõi của tổ chức này. Từ một nước nhận viện trợ của Liên hợp quốc, Việt Nam chuyển mình, từng bước trở thành thành viên tin cậy, hiệu quả của Liên hợp quốc, là nước đóng góp lớn thứ 49 cho ngân sách của Liên hợp quốc, tham gia ngày càng sâu rộng trên cả ba trụ cột chính: hòa bình - an ninh, hợp tác phát triển và quyền con người.</t>
-  </si>
-  <si>
-    <t>Từ tro tàn của Chiến tranh thế giới lần thứ hai, ngày 24-10-1945, Liên hợp quốc được thành lập với sứ mệnh cao cả là “cứu các thế hệ mai sau khỏi thảm họa chiến tranh đã gây ra đau thương tột cùng cho nhân loại hai lần trong một đời người”. Sự ra đời của Liên hợp quốc là bước ngoặt quan trọng trong lịch sử với cam kết ngăn chặn, loại bỏ các mối đe dọa đối với hòa bình và an ninh quốc tế, các hành vi xâm lược, thúc đẩy giải quyết tranh chấp bằng biện pháp hòa bình.
-Hiến chương Liên hợp quốc là văn kiện nền tảng đặt ra các nguyên tắc cốt lõi mà mọi quốc gia thành viên phải tuân thủ, là khuôn khổ điều chỉnh hành vi của các quốc gia trong suốt gần 80 năm qua và tạo nền tảng cho hệ thống luật pháp quốc tế hiện đại. Đặc biệt, lần đầu tiên trong lịch sử nhân loại, hành vi đe dọa sử dụng vũ lực hoặc sử dụng vũ lực nhằm xâm phạm sự toàn vẹn lãnh thổ và độc lập chính trị của một quốc gia hoặc gây tổn hại đến hòa bình và an ninh quốc tế, bị nghiêm cấm theo Điều 2 của Hiến chương Liên hợp quốc.</t>
-  </si>
-  <si>
-    <t>Hội nghị I-an-ta diễn ra từ ngày 4 đến ngày 11-2-1945 đã đưa ra những quyết định quan trọng về việc kết thúc chiến tranh và thỏa thuận về việc đóng quân, phân chia phạm vi ảnh hưởng ở châu Âu và châu Á. Những quyết định này cùng với những thỏa thuận sau đó của các cường quốc đã trở thành khuôn khổ cho sự thiết lập trật tự thế giới mới, gọi là Trật tự thế giới hai cực I-an-ta. Trong quá trình tồn tại, trật tự này được định hình với sự thiết lập các khối quân sự đối đầu nhau, tiêu biểu là Tổ chức Hiệp ước Bắc Đại Tây Dương (NATO) và Tổ chức Hiệp ước Vác-sa-va</t>
-  </si>
-  <si>
-    <t>Tuyên bố Kuala Lupur về việc hình thành Cộng đồng ASEAN vào ngày 31-12-2015 khẳng định cam kết của các nước thành viên đối với Hiến chương ASEAN, phản ánh mong muốn và ý chí tập thể nhằm chung sống trong một khu vực hòa bình, an ninh và ổn định dài lâu, tăng trưởng kinh tế bền vững, thịnh vượng chung và tiến bộ xã hội,… đánh dấu một bước ngoặt lịch sử mới trong quá trình phát triển của ASEAN, phản ánh được sự lớn mạnh của ASEAN sau gần 48 năm hình thành, phát triển và vươn lên trở thành một Cộng đồng liên kết chặt chẽ trên cả 3 trụ cột là chính trị - an ninh, kinh tế và văn hóa - xã hội với vị thế ngày càng cao ở cả khu vực và thế giới.
-Các nhà lãnh đạo ASEAN coi việc hình thành Cộng đồng ASEAN 2015 là dấu mốc lịch sử trong tiến trình liên kết khu vực, đánh dấu bước chuyển mình chiến lược của ASEAN và khởi đầu cho một giai đoạn phát triển mới ở tầm cao hơn của ASEAN. Đồng thời nhấn mạnh, xây dựng Cộng đồng ASEAN là một tiến trình liên tục; nhất trí rằng, ASEAN cần tiếp tục củng cố và đưa liên kết ASEAN lên tầm cao mới trên cơ sở tiếp nối và phát huy các thành tựu đã đạt được.
-Theo đó, các nhà lãnh đạo ASEAN đã thông qua Tầm nhìn Cộng đồng ASEAN 2025 và ba Kế hoạch Tổng thể triển khai Tầm nhìn trên 3 trụ cột với chủ đề “ASEAN 2025: cùng vững vàng tiến bước” định hướng và tạo cơ sở, khuôn khổ cho liên kết của ASEAN trong mười năm tới. Các nhà lãnh đạo cam kết triển khai hiệu quả các văn kiện này; đồng thời nhất trí, cần tiếp tục triển khai hiệu quả Kế hoạch Tổng thể về Kết nối và Sáng kiến Liên kết ASEAN về thu hẹp khoảng cách phát triển để hỗ trợ cho tiến trình xây dựng Cộng đồng.</t>
-  </si>
-  <si>
     <t>Tài liệu bổ sung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“Chiến tranh lạnh” kết thúc, trật tự hai cực biểu hiện cuộc đối đầu Đông – Tây khốc liệt của thế giới đã đi đến điểm kết. Song, trật tự thế giới mới vẫn còn đang trong quá trình hình thành. Dựa vào thực lực kinh tế, chính trị và quân sự của mình, Mỹ không từ bỏ mục đích bá chủ thế giới. Tuy nhiên, sự phát triển không ngừng của Nhật Bản, Tây Âu; sự vươn lên mạnh mẽ của Trung Quốc; những cuộc đấu tranh mạnh mẽ nhằm củng cố, bảo vệ độc lập, chủ quyền của các nước thuộc “thế giới thứ ba” dưới nhiều hình thức, biện pháp để chống lại sự can thiệp và ảnh hưởng của các nước lớn… đã tạo ra những tương quan lực lượng không nhỏ đối với Mỹ. Điều này cho thấy, thế giới hậu lưỡng cực đang hướng tới xác lập một trật tự mới với nhiều hướng khác nhau: đơn cực, đa cực, nhất siêu đa cường...
-Sự kết thúc của “Chiến tranh lạnh” tuy không mở ra kỷ nguyên mới hòa bình và thịnh vượng như nhân loại tiến bộ mong đợi vì những xung đột sắc tộc, mâu thuẫn tôn giáo và các cuộc chiến tranh cục bộ ở nhiều khu vực vẫn diễn ra triền miên, song đã tạo ra những điều kiện khiến cho xu thế hòa dịu, hòa hoãn trở nên chiếm ưu thế trong quan hệ giữa các quốc gia, dân tộc trên thế giới; tạo những tiền đề cho đa cực hóa các mối quan hệ- một điều kiện quan trọng dẫn đến hình thành xu thế đa dạng hóa, đa phương hóa, hội nhập khu vực và quốc tế trong quan hệ quốc tế hiện nay.
-https://www.tapchicongsan.org.vn/web/guest/nghien-cu/-/2018/3089/xu-the-da-dang-hoa%2C-da-phuong-hoa%2C-hoi-nhap-khu-vuc-va-quoc-te-hien-nay.aspx </t>
   </si>
   <si>
     <t>Bài 1. Liên Hợp Quốc
@@ -1202,6 +1132,30 @@
 Tìm hiểu thông tin từ sách, báo, internet và chia sẻ với bạn về những đóng góp, hỗ trợ của Liên hợp quốc đối với Việt Nam.
 12
 ==End of OCR for page 7==</t>
+  </si>
+  <si>
+    <t>Tư liệu 1. “Về quyền con người, Liên hợp quốc đóng vai trò tiên phong trong đàm phán và xây dựng các văn kiện quốc tế quan trọng, trong đó có Tuyên ngôn Nhân quyền thế giới (năm 1948), Công ước quốc tế về các quyền kinh tế, xã hội và văn hoá (năm 1966), Công ước quốc tế về các quyền dân sự và chính trị (năm 1966) [...] Liên hợp quốc cũng đặc biệt chú trọng đến việc bảo đảm thực hiện quyền con người thông qua các cơ chế, như Hội đồng Nhân quyền Liên hợp quốc, các báo cáo viên đặc biệt của Liên hợp quốc cùng hệ thống cơ quan công ước quốc tế về quyền con người.”
+(“Quan hệ Việt Nam - Liên hợp quốc: Khởi đầu hợp tác mới vì một tương lai tốt đẹp của nhân loại”, Tạp chí Cộng sản, đăng ngày 21/09/2024, https://www.tapchicongsan.org.vn)
+Tư liệu 2. “Việt Nam đã 2 lần trúng cử vào Hội đồng Nhân quyền Liên Hiệp Quốc. Lần đầu tiên vào năm 2013, Việt Nam trúng cử vào hội đồng nhiệm kỳ 2014 - 2016. Ngày 11/10/2022, Việt Nam trúng cử trở thành thành viên của Hội đồng Nhân quyền Liên Hiệp Quốc nhiệm kỳ 2023 - 2025.”
+(“Việt Nam tái ứng cử Hội đồng Nhân quyền Liên Hiệp Quốc nhiệm kỳ 2026 - 2028”, Báo Tuổi trẻ online, đăng ngày 13/12/2024, https://tuoitre.vn)</t>
+  </si>
+  <si>
+    <t>“Ở “Trật tự hai cực I-an-ta”, Liên Xô đã đạt được 3 mục tiêu cơ bản: Bảo vệ vững chắc sự tồn tại và phát triển của đất nước Xô viết; thu hồi lại những đất đai của đế quốc Nga trước đây (kể từ chiến tranh Nga - Nhật 1904 - 1905 đến chiến tranh chống ngoại xâm và nội phản 1918 - 1920); mở rộng phạm vi ảnh hưởng ở châu Âu và châu Á, qua đó thiết lập một vành đai an toàn bao quanh phía tây, đông và nam Liên Xô. Còn Mỹ, với trật tự thế giới mới này, Mỹ đã khống chế được Tây Âu, Nhật Bản, chi phối cục diện thế giới. Mặt khác, sự thoả thuận giữa ba cường quốc ở Hội nghị I-an-ta đã xâm phạm đến chủ quyền, lãnh thổ và lợi ích của nhân dân nhiều nước”.
+(Nguyễn Anh Thái (Chủ biên), Lịch sử thế giới hiện đại (1917 - 1995), NXB Giáo dục, 2006, tr. 234)</t>
+  </si>
+  <si>
+    <t>“Cục diện thế giới hiện nay (từ đầu thế kỉ XXI đến nay), vừa chứa đựng một số đặc điểm kế thừa từ các cục diện trước đó, vừa có biểu hiện mới của đặc điểm cũ và cả những đặc điểm mới. Rõ nhất là đặc điểm đa cực, đa trung tâm: hiển nhiên đã từng xuất hiện từ những năm cuối thế kỉ XX, nhưng từ khi Trung Quốc trở thành nền kinh tế thứ hai thế giới (2010), tương quan quyền lực giữa các cực, các trung tâm đã khác hẳn, tạo cơ sở cho quyết định chấm dứt thời kì “giấu mình, chờ thời” (năm 2017) của các cường quốc đang trỗi dậy. Cuộc chiến tranh chiến lược Mỹ - Trung ở khu vực châu Á - Thái Bình Dương trong những năm vừa qua có thể được xem như đặc điểm mới của cục diện thế giới hiện nay, mặc dù đã manh nha từ nhiều năm trước.”
+(Nguyễn Viết Thảo, “Bối cảnh hình thành và đặc điểm nổi bật của cục diện thế giới hiện nay”, Tạp chí Lí luận Chính trị số 541 (3/2023), tr. 151)</t>
+  </si>
+  <si>
+    <t>Cho bảng thông tin sau:
+Thời gian 	Nội dung
+Ngày 8/8/1967	Tổ chức ASEAN được thành lập tại Băng Cốc (Thái Lan) với 5 nước sáng lập
+Năm 1971	ASEAN ra Tuyên bố về khu vực hoà bình, tự do và trung lập.
+Năm 1976	Hiệp ước Ba-li được kí kết, đề ra những nguyên tắc cơ bản trong quan hệ giữa các nước ASEAN.
+Năm 1984	Bru-nây trở thành thành viên thứ 6 của ASEAN.
+1995 - 1999	Việt Nam, Lào, Mi-an-ma, Cam-pu-chia gia nhập ASEAN.
+Năm 2007	Hiến chương ASEAN được thông qua.</t>
   </si>
 </sst>
 </file>
@@ -1467,66 +1421,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1541,6 +1435,66 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1902,43 +1856,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39" t="s">
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39" t="s">
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="P1" s="28"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="P1" s="27"/>
     </row>
     <row r="2" spans="2:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="24"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="22"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="31"/>
       <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1966,18 +1920,18 @@
       <c r="N2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
     </row>
     <row r="3" spans="2:16" ht="119.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="35">
+      <c r="B3" s="44">
         <v>1</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="41" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>46</v>
@@ -1995,16 +1949,14 @@
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
-      <c r="O3" s="44" t="s">
-        <v>70</v>
-      </c>
-      <c r="P3" s="44" t="s">
-        <v>71</v>
-      </c>
+      <c r="O3" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="P3" s="24"/>
     </row>
     <row r="4" spans="2:16" ht="152.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="36"/>
-      <c r="C4" s="33"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="42"/>
       <c r="D4" s="9" t="s">
         <v>66</v>
       </c>
@@ -2024,16 +1976,14 @@
       <c r="L4" s="8"/>
       <c r="M4" s="8"/>
       <c r="N4" s="8"/>
-      <c r="O4" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="P4" s="44" t="s">
+      <c r="O4" s="24" t="s">
         <v>73</v>
       </c>
+      <c r="P4" s="24"/>
     </row>
     <row r="5" spans="2:16" ht="95.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="36"/>
-      <c r="C5" s="33"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="42"/>
       <c r="D5" s="9" t="s">
         <v>67</v>
       </c>
@@ -2055,14 +2005,14 @@
       <c r="L5" s="8"/>
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
-      <c r="O5" s="44" t="s">
+      <c r="O5" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="P5" s="44"/>
+      <c r="P5" s="24"/>
     </row>
     <row r="6" spans="2:16" ht="168" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="36"/>
-      <c r="C6" s="33"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="42"/>
       <c r="D6" s="10" t="s">
         <v>68</v>
       </c>
@@ -2084,16 +2034,14 @@
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
-      <c r="O6" s="44" t="s">
+      <c r="O6" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="P6" s="44" t="s">
-        <v>76</v>
-      </c>
+      <c r="P6" s="24"/>
     </row>
     <row r="7" spans="2:16" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="37"/>
-      <c r="C7" s="34"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="43"/>
       <c r="D7" s="10" t="s">
         <v>69</v>
       </c>
@@ -2113,18 +2061,18 @@
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
-      <c r="O7" s="44"/>
-      <c r="P7" s="44"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24"/>
     </row>
     <row r="8" spans="2:16" ht="172.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="35">
+      <c r="B8" s="44">
         <v>2</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="41" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>51</v>
@@ -2144,16 +2092,12 @@
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
-      <c r="O8" s="44" t="s">
-        <v>77</v>
-      </c>
-      <c r="P8" s="44" t="s">
-        <v>78</v>
-      </c>
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
     </row>
     <row r="9" spans="2:16" ht="246" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="36"/>
-      <c r="C9" s="33"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="42"/>
       <c r="D9" s="9" t="s">
         <v>66</v>
       </c>
@@ -2175,14 +2119,12 @@
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
-      <c r="O9" s="44" t="s">
-        <v>79</v>
-      </c>
-      <c r="P9" s="44"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
     </row>
     <row r="10" spans="2:16" ht="221.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="36"/>
-      <c r="C10" s="33"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="42"/>
       <c r="D10" s="9" t="s">
         <v>67</v>
       </c>
@@ -2204,14 +2146,12 @@
       <c r="L10" s="8"/>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
-      <c r="O10" s="45" t="s">
-        <v>82</v>
-      </c>
-      <c r="P10" s="44"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="24"/>
     </row>
     <row r="11" spans="2:16" ht="251.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="36"/>
-      <c r="C11" s="33"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="42"/>
       <c r="D11" s="10" t="s">
         <v>68</v>
       </c>
@@ -2233,14 +2173,12 @@
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
-      <c r="O11" s="44" t="s">
-        <v>80</v>
-      </c>
-      <c r="P11" s="44"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
     </row>
     <row r="12" spans="2:16" ht="122.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="37"/>
-      <c r="C12" s="34"/>
+      <c r="B12" s="46"/>
+      <c r="C12" s="43"/>
       <c r="D12" s="10" t="s">
         <v>69</v>
       </c>
@@ -2258,18 +2196,18 @@
       <c r="L12" s="8"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
-      <c r="O12" s="44"/>
-      <c r="P12" s="44"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="24"/>
     </row>
     <row r="13" spans="2:16" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="35">
+      <c r="B13" s="44">
         <v>3</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="41" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>55</v>
@@ -2287,12 +2225,12 @@
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
-      <c r="O13" s="44"/>
-      <c r="P13" s="44"/>
+      <c r="O13" s="24"/>
+      <c r="P13" s="24"/>
     </row>
     <row r="14" spans="2:16" ht="86.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="36"/>
-      <c r="C14" s="33"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="42"/>
       <c r="D14" s="9" t="s">
         <v>66</v>
       </c>
@@ -2310,12 +2248,12 @@
       <c r="L14" s="8"/>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
-      <c r="O14" s="44"/>
-      <c r="P14" s="44"/>
+      <c r="O14" s="24"/>
+      <c r="P14" s="24"/>
     </row>
     <row r="15" spans="2:16" ht="107.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="36"/>
-      <c r="C15" s="33"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="42"/>
       <c r="D15" s="9" t="s">
         <v>67</v>
       </c>
@@ -2335,12 +2273,12 @@
       <c r="L15" s="8"/>
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
-      <c r="O15" s="44"/>
-      <c r="P15" s="44"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="24"/>
     </row>
     <row r="16" spans="2:16" ht="107.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="36"/>
-      <c r="C16" s="33"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="42"/>
       <c r="D16" s="10" t="s">
         <v>68</v>
       </c>
@@ -2360,12 +2298,12 @@
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
-      <c r="O16" s="44"/>
-      <c r="P16" s="44"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
     </row>
     <row r="17" spans="2:16" ht="91.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="37"/>
-      <c r="C17" s="34"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="43"/>
       <c r="D17" s="10" t="s">
         <v>69</v>
       </c>
@@ -2383,8 +2321,8 @@
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
-      <c r="O17" s="44"/>
-      <c r="P17" s="44"/>
+      <c r="O17" s="24"/>
+      <c r="P17" s="24"/>
     </row>
     <row r="18" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="12">
@@ -2402,8 +2340,8 @@
       <c r="L18" s="8"/>
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
-      <c r="O18" s="41"/>
-      <c r="P18" s="41"/>
+      <c r="O18" s="21"/>
+      <c r="P18" s="21"/>
     </row>
     <row r="19" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="12">
@@ -2421,8 +2359,8 @@
       <c r="L19" s="8"/>
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
-      <c r="O19" s="41"/>
-      <c r="P19" s="41"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
     </row>
     <row r="20" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="12">
@@ -2440,8 +2378,8 @@
       <c r="L20" s="8"/>
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
-      <c r="O20" s="41"/>
-      <c r="P20" s="41"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="21"/>
     </row>
     <row r="21" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="12">
@@ -2459,8 +2397,8 @@
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
-      <c r="O21" s="41"/>
-      <c r="P21" s="41"/>
+      <c r="O21" s="21"/>
+      <c r="P21" s="21"/>
     </row>
     <row r="22" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="12">
@@ -2478,8 +2416,8 @@
       <c r="L22" s="8"/>
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
-      <c r="O22" s="42"/>
-      <c r="P22" s="43"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="23"/>
     </row>
     <row r="23" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="12">
@@ -2497,8 +2435,8 @@
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
-      <c r="O23" s="42"/>
-      <c r="P23" s="43"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="23"/>
     </row>
     <row r="24" spans="2:16" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="12">
@@ -2516,11 +2454,11 @@
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
-      <c r="O24" s="42"/>
-      <c r="P24" s="43"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="23"/>
     </row>
     <row r="25" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="27" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="17" t="s">
@@ -2558,11 +2496,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O25" s="46"/>
-      <c r="P25" s="46"/>
+      <c r="O25" s="26"/>
+      <c r="P25" s="26"/>
     </row>
     <row r="26" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="28"/>
+      <c r="B26" s="27"/>
       <c r="C26" s="18" t="s">
         <v>11</v>
       </c>
@@ -2604,71 +2542,66 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O26" s="46"/>
-      <c r="P26" s="46"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
     </row>
     <row r="27" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="28"/>
+      <c r="B27" s="27"/>
       <c r="C27" s="18" t="s">
         <v>12</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="20"/>
-      <c r="F27" s="29">
+      <c r="F27" s="38">
         <v>24</v>
       </c>
-      <c r="G27" s="30"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="29">
+      <c r="G27" s="39"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="38">
         <f>I25+J25+K25</f>
         <v>16</v>
       </c>
-      <c r="J27" s="30"/>
-      <c r="K27" s="31"/>
-      <c r="L27" s="29">
+      <c r="J27" s="39"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="38">
         <f>L25+M25+N25</f>
         <v>0</v>
       </c>
-      <c r="M27" s="30"/>
-      <c r="N27" s="31"/>
-      <c r="O27" s="46"/>
-      <c r="P27" s="46"/>
+      <c r="M27" s="39"/>
+      <c r="N27" s="40"/>
+      <c r="O27" s="26"/>
+      <c r="P27" s="26"/>
     </row>
     <row r="28" spans="2:16" s="1" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="28"/>
+      <c r="B28" s="27"/>
       <c r="C28" s="18" t="s">
         <v>13</v>
       </c>
       <c r="D28" s="20"/>
       <c r="E28" s="20"/>
-      <c r="F28" s="25">
+      <c r="F28" s="35">
         <f>(F27/40)*100</f>
         <v>60</v>
       </c>
-      <c r="G28" s="26"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="25">
+      <c r="G28" s="36"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="35">
         <f>(I27/40)*100</f>
         <v>40</v>
       </c>
-      <c r="J28" s="26"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="25">
+      <c r="J28" s="36"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="35">
         <f>(L27/40)*100</f>
         <v>0</v>
       </c>
-      <c r="M28" s="26"/>
-      <c r="N28" s="27"/>
-      <c r="O28" s="46"/>
-      <c r="P28" s="46"/>
+      <c r="M28" s="36"/>
+      <c r="N28" s="37"/>
+      <c r="O28" s="26"/>
+      <c r="P28" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="O1:P2"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
@@ -2685,6 +2618,11 @@
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="B13:B17"/>
+    <mergeCell ref="O1:P2"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>